<commit_message>
updated logo and app icon
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Markus/Documents/Arbeit/Inschriftenschluessel/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DB98674-A200-DF4A-B28B-FF015CF7E6B7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35661E5B-161B-C949-9164-F5F6295C330C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="460" yWindow="500" windowWidth="20220" windowHeight="16120" activeTab="3" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
+    <workbookView xWindow="460" yWindow="500" windowWidth="20220" windowHeight="16120" activeTab="5" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
   </bookViews>
   <sheets>
     <sheet name="pages" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
added tutorial of adding to home-screen
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Markus/Documents/Arbeit/Inschriftenschluessel/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A08C6DEA-2EDE-FF46-AF23-3FE582C1D426}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F52C211B-54B0-5E43-9633-E2CDD32BFAC2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19720" activeTab="4" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
+    <workbookView xWindow="6540" yWindow="500" windowWidth="22260" windowHeight="16200" activeTab="6" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
   </bookViews>
   <sheets>
     <sheet name="pages" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="slot_content" sheetId="6" r:id="rId4"/>
     <sheet name="glyphlines" sheetId="5" r:id="rId5"/>
     <sheet name="tables" sheetId="4" r:id="rId6"/>
+    <sheet name="tutorial_steps" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7929" uniqueCount="1645">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7957" uniqueCount="1666">
   <si>
     <t>page_id</t>
   </si>
@@ -4987,6 +4988,69 @@
   <si>
     <t>- Lapp, Günther. 1986. Die Opferformel des Alten Reiches: unter Berücksichtigung einiger späterer Formen. Sonderschrift, Deutsches Archäologisches Institut, Abteilung Kairo 21. Philipp von Zabern.</t>
   </si>
+  <si>
+    <t>platform</t>
+  </si>
+  <si>
+    <t>image</t>
+  </si>
+  <si>
+    <t>caption</t>
+  </si>
+  <si>
+    <t>ios</t>
+  </si>
+  <si>
+    <t>Öffne die Webseite in Safari.</t>
+  </si>
+  <si>
+    <t>Tippe unten auf das Teilen-Symbol.</t>
+  </si>
+  <si>
+    <t>Wähle „Zum Home-Bildschirm“.</t>
+  </si>
+  <si>
+    <t>Bestätige mit „Hinzufügen“.</t>
+  </si>
+  <si>
+    <t>android</t>
+  </si>
+  <si>
+    <t>assets/tutorial/android-01.webp</t>
+  </si>
+  <si>
+    <t>Öffne die Webseite in Chrome.</t>
+  </si>
+  <si>
+    <t>assets/tutorial/android-02.webp</t>
+  </si>
+  <si>
+    <t>Öffne das Browser-Menü.</t>
+  </si>
+  <si>
+    <t>assets/tutorial/android-03.webp</t>
+  </si>
+  <si>
+    <t>Wähle „App installieren“.</t>
+  </si>
+  <si>
+    <t>assets/tutorial/android-04.webp</t>
+  </si>
+  <si>
+    <t>Bestätige die Installation.</t>
+  </si>
+  <si>
+    <t>assets/tutorial/ios_01.webp</t>
+  </si>
+  <si>
+    <t>assets/tutorial/ios_02.webp</t>
+  </si>
+  <si>
+    <t>assets/tutorial/ios_03.webp</t>
+  </si>
+  <si>
+    <t>assets/tutorial/ios_04.webp</t>
+  </si>
 </sst>
 </file>
 
@@ -4995,7 +5059,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0000"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -5048,6 +5112,25 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -5126,7 +5209,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -5265,6 +5348,9 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -6152,7 +6238,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" s="14" customFormat="1" ht="102">
+    <row r="3" spans="1:6" s="14" customFormat="1" ht="119">
       <c r="A3" s="14" t="s">
         <v>9</v>
       </c>
@@ -6636,7 +6722,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="37" spans="1:6" s="24" customFormat="1" ht="34">
+    <row r="37" spans="1:6" s="24" customFormat="1" ht="51">
       <c r="A37" s="24" t="s">
         <v>65</v>
       </c>
@@ -6795,7 +6881,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="48" spans="1:6" s="27" customFormat="1" ht="85">
+    <row r="48" spans="1:6" s="27" customFormat="1" ht="102">
       <c r="A48" s="27" t="s">
         <v>66</v>
       </c>
@@ -6872,7 +6958,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="1:6" s="30" customFormat="1" ht="136">
+    <row r="54" spans="1:6" s="30" customFormat="1" ht="153">
       <c r="A54" s="30" t="s">
         <v>67</v>
       </c>
@@ -9197,7 +9283,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="138" spans="1:11" ht="204">
+    <row r="138" spans="1:11" ht="221">
       <c r="A138" s="13" t="s">
         <v>1257</v>
       </c>
@@ -22598,7 +22684,7 @@
         <v>1594</v>
       </c>
       <c r="L286" s="57" t="str">
-        <f>_xlfn.TEXTJOIN("", TRUE, D286:K286)</f>
+        <f t="shared" ref="L286:L291" si="50">_xlfn.TEXTJOIN("", TRUE, D286:K286)</f>
         <v>02_Slots/Datum/02_Monat/01_Abd/0001_Abd_01.png</v>
       </c>
     </row>
@@ -22622,7 +22708,7 @@
         <v>1595</v>
       </c>
       <c r="L287" s="57" t="str">
-        <f>_xlfn.TEXTJOIN("", TRUE, D287:K287)</f>
+        <f t="shared" si="50"/>
         <v>02_Slots/Datum/02_Monat/01_Abd/0010_Abd_02.png</v>
       </c>
     </row>
@@ -22655,7 +22741,7 @@
         <v>1092</v>
       </c>
       <c r="L288" s="57" t="str">
-        <f>_xlfn.TEXTJOIN("", TRUE, D288:K288)</f>
+        <f t="shared" si="50"/>
         <v>02_Slots/Datum/02_Monat/01_Abd/0020_Abd_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -22688,7 +22774,7 @@
         <v>1092</v>
       </c>
       <c r="L289" s="57" t="str">
-        <f>_xlfn.TEXTJOIN("", TRUE, D289:K289)</f>
+        <f t="shared" si="50"/>
         <v>02_Slots/Datum/02_Monat/01_Abd/0030_Abd_AR_02.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -22721,7 +22807,7 @@
         <v>1092</v>
       </c>
       <c r="L290" s="57" t="str">
-        <f>_xlfn.TEXTJOIN("", TRUE, D290:K290)</f>
+        <f t="shared" si="50"/>
         <v>02_Slots/Datum/02_Monat/01_Abd/0040_Abd_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -22754,7 +22840,7 @@
         <v>1092</v>
       </c>
       <c r="L291" s="57" t="str">
-        <f>_xlfn.TEXTJOIN("", TRUE, D291:K291)</f>
+        <f t="shared" si="50"/>
         <v>02_Slots/Datum/02_Monat/01_Abd/0050_Abd_Gr_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -22851,7 +22937,7 @@
         <v>111</v>
       </c>
       <c r="L297" s="57" t="str">
-        <f t="shared" ref="L297" si="50">_xlfn.TEXTJOIN("", TRUE, D297:J297)</f>
+        <f t="shared" ref="L297" si="51">_xlfn.TEXTJOIN("", TRUE, D297:J297)</f>
         <v>02_Slots/Datum/02_Monat/0010_tpy_01.png</v>
       </c>
     </row>
@@ -23022,7 +23108,7 @@
         <v>1384</v>
       </c>
       <c r="L310" s="57" t="str">
-        <f t="shared" ref="L310:L314" si="51">_xlfn.TEXTJOIN("", TRUE, D310:K310)</f>
+        <f t="shared" ref="L310:L314" si="52">_xlfn.TEXTJOIN("", TRUE, D310:K310)</f>
         <v>02_Slots/Datum/03_Jahreszeiten/01_Ax.t/0001_Ax.t_01.png</v>
       </c>
     </row>
@@ -23046,7 +23132,7 @@
         <v>1385</v>
       </c>
       <c r="L311" s="57" t="str">
-        <f t="shared" si="51"/>
+        <f t="shared" si="52"/>
         <v>02_Slots/Datum/03_Jahreszeiten/01_Ax.t/0010_Ax.t_02.png</v>
       </c>
     </row>
@@ -23070,7 +23156,7 @@
         <v>1386</v>
       </c>
       <c r="L312" s="57" t="str">
-        <f t="shared" si="51"/>
+        <f t="shared" si="52"/>
         <v>02_Slots/Datum/03_Jahreszeiten/01_Ax.t/0020_Ax.t_03.png</v>
       </c>
     </row>
@@ -23094,7 +23180,7 @@
         <v>1387</v>
       </c>
       <c r="L313" s="57" t="str">
-        <f t="shared" si="51"/>
+        <f t="shared" si="52"/>
         <v>02_Slots/Datum/03_Jahreszeiten/01_Ax.t/0030_Ax.t_04.png</v>
       </c>
     </row>
@@ -23127,7 +23213,7 @@
         <v>1092</v>
       </c>
       <c r="L314" s="57" t="str">
-        <f t="shared" si="51"/>
+        <f t="shared" si="52"/>
         <v>02_Slots/Datum/03_Jahreszeiten/01_Ax.t/0040_Ax.t_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -23221,7 +23307,7 @@
         <v>1389</v>
       </c>
       <c r="L320" s="57" t="str">
-        <f t="shared" ref="L320:L325" si="52">_xlfn.TEXTJOIN("", TRUE, D320:K320)</f>
+        <f t="shared" ref="L320:L325" si="53">_xlfn.TEXTJOIN("", TRUE, D320:K320)</f>
         <v>02_Slots/Datum/03_Jahreszeiten/02_pr.t/0001_pr.t_01.png</v>
       </c>
     </row>
@@ -23245,7 +23331,7 @@
         <v>1390</v>
       </c>
       <c r="L321" s="57" t="str">
-        <f t="shared" si="52"/>
+        <f t="shared" si="53"/>
         <v>02_Slots/Datum/03_Jahreszeiten/02_pr.t/0010_pr.t_02.png</v>
       </c>
     </row>
@@ -23278,7 +23364,7 @@
         <v>1092</v>
       </c>
       <c r="L322" s="57" t="str">
-        <f t="shared" si="52"/>
+        <f t="shared" si="53"/>
         <v>02_Slots/Datum/03_Jahreszeiten/02_pr.t/0020_pr.t_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -23311,7 +23397,7 @@
         <v>1092</v>
       </c>
       <c r="L323" s="57" t="str">
-        <f t="shared" si="52"/>
+        <f t="shared" si="53"/>
         <v>02_Slots/Datum/03_Jahreszeiten/02_pr.t/0030_pr.t_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -23344,7 +23430,7 @@
         <v>1092</v>
       </c>
       <c r="L324" s="57" t="str">
-        <f t="shared" si="52"/>
+        <f t="shared" si="53"/>
         <v>02_Slots/Datum/03_Jahreszeiten/02_pr.t/0040_pr.t_Sp_01.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -23377,7 +23463,7 @@
         <v>1092</v>
       </c>
       <c r="L325" s="57" t="str">
-        <f t="shared" si="52"/>
+        <f t="shared" si="53"/>
         <v>02_Slots/Datum/03_Jahreszeiten/02_pr.t/0050_pr.t_Gr_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -23471,7 +23557,7 @@
         <v>1395</v>
       </c>
       <c r="L331" s="57" t="str">
-        <f t="shared" ref="L331:L340" si="53">_xlfn.TEXTJOIN("", TRUE, D331:K331)</f>
+        <f t="shared" ref="L331:L340" si="54">_xlfn.TEXTJOIN("", TRUE, D331:K331)</f>
         <v>02_Slots/Datum/03_Jahreszeiten/03_Smw/0001_Smw_01.png</v>
       </c>
     </row>
@@ -23495,7 +23581,7 @@
         <v>1396</v>
       </c>
       <c r="L332" s="57" t="str">
-        <f t="shared" si="53"/>
+        <f t="shared" si="54"/>
         <v>02_Slots/Datum/03_Jahreszeiten/03_Smw/0010_Smw_02.png</v>
       </c>
     </row>
@@ -23519,7 +23605,7 @@
         <v>1397</v>
       </c>
       <c r="L333" s="57" t="str">
-        <f t="shared" si="53"/>
+        <f t="shared" si="54"/>
         <v>02_Slots/Datum/03_Jahreszeiten/03_Smw/0020_Smw_03.png</v>
       </c>
     </row>
@@ -23552,7 +23638,7 @@
         <v>1092</v>
       </c>
       <c r="L334" s="57" t="str">
-        <f t="shared" si="53"/>
+        <f t="shared" si="54"/>
         <v>02_Slots/Datum/03_Jahreszeiten/03_Smw/0030_Smw_D.20_01.png &lt;sup&gt;(D.20)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -23585,7 +23671,7 @@
         <v>1092</v>
       </c>
       <c r="L335" s="57" t="str">
-        <f t="shared" si="53"/>
+        <f t="shared" si="54"/>
         <v>02_Slots/Datum/03_Jahreszeiten/03_Smw/0040_Smw_Sp_Gr_Abk_01.png &lt;sup&gt;(Sp.–Gr.; Abk.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -23618,7 +23704,7 @@
         <v>1092</v>
       </c>
       <c r="L336" s="57" t="str">
-        <f t="shared" si="53"/>
+        <f t="shared" si="54"/>
         <v>02_Slots/Datum/03_Jahreszeiten/03_Smw/0050_Smw_Sp_Gr_Abk_02.png &lt;sup&gt;(Sp.–Gr.; Abk.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -23651,7 +23737,7 @@
         <v>1092</v>
       </c>
       <c r="L337" s="57" t="str">
-        <f t="shared" si="53"/>
+        <f t="shared" si="54"/>
         <v>02_Slots/Datum/03_Jahreszeiten/03_Smw/0060_Smw_Sp_Gr_Abk_03.png &lt;sup&gt;(Sp.–Gr.; Abk.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -23684,7 +23770,7 @@
         <v>1092</v>
       </c>
       <c r="L338" s="57" t="str">
-        <f t="shared" si="53"/>
+        <f t="shared" si="54"/>
         <v>02_Slots/Datum/03_Jahreszeiten/03_Smw/0070_Smw_Gr_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -23717,7 +23803,7 @@
         <v>1092</v>
       </c>
       <c r="L339" s="57" t="str">
-        <f t="shared" si="53"/>
+        <f t="shared" si="54"/>
         <v>02_Slots/Datum/03_Jahreszeiten/03_Smw/0080_Smw_Gr_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -23750,7 +23836,7 @@
         <v>1092</v>
       </c>
       <c r="L340" s="57" t="str">
-        <f t="shared" si="53"/>
+        <f t="shared" si="54"/>
         <v>02_Slots/Datum/03_Jahreszeiten/03_Smw/0090_Smw_Gr_03.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -23918,7 +24004,7 @@
         <v>1410</v>
       </c>
       <c r="L353" s="57" t="str">
-        <f t="shared" ref="L353:L359" si="54">_xlfn.TEXTJOIN("", TRUE, D353:K353)</f>
+        <f t="shared" ref="L353:L359" si="55">_xlfn.TEXTJOIN("", TRUE, D353:K353)</f>
         <v>02_Slots/Datum/04_Tag/0001_sw_01.png</v>
       </c>
     </row>
@@ -23942,7 +24028,7 @@
         <v>1411</v>
       </c>
       <c r="L354" s="57" t="str">
-        <f t="shared" si="54"/>
+        <f t="shared" si="55"/>
         <v>02_Slots/Datum/04_Tag/0010_sw_02.png</v>
       </c>
     </row>
@@ -23975,7 +24061,7 @@
         <v>1092</v>
       </c>
       <c r="L355" s="57" t="str">
-        <f t="shared" si="54"/>
+        <f t="shared" si="55"/>
         <v>02_Slots/Datum/04_Tag/0020_sw_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -24008,7 +24094,7 @@
         <v>1092</v>
       </c>
       <c r="L356" s="57" t="str">
-        <f t="shared" si="54"/>
+        <f t="shared" si="55"/>
         <v>02_Slots/Datum/04_Tag/0030_sw_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -24041,7 +24127,7 @@
         <v>1092</v>
       </c>
       <c r="L357" s="57" t="str">
-        <f t="shared" si="54"/>
+        <f t="shared" si="55"/>
         <v>02_Slots/Datum/04_Tag/0040_sw_Sp_01.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -24074,7 +24160,7 @@
         <v>1092</v>
       </c>
       <c r="L358" s="57" t="str">
-        <f t="shared" si="54"/>
+        <f t="shared" si="55"/>
         <v>02_Slots/Datum/04_Tag/0050_sw_Sp_02.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -24107,7 +24193,7 @@
         <v>1092</v>
       </c>
       <c r="L359" s="57" t="str">
-        <f t="shared" si="54"/>
+        <f t="shared" si="55"/>
         <v>02_Slots/Datum/04_Tag/0060_sw_Sp_03.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -24225,7 +24311,7 @@
         <v>1409</v>
       </c>
       <c r="L366" s="57" t="str">
-        <f t="shared" ref="L366:L368" si="55">_xlfn.TEXTJOIN("", TRUE, D366:K366)</f>
+        <f t="shared" ref="L366:L368" si="56">_xlfn.TEXTJOIN("", TRUE, D366:K366)</f>
         <v>02_Slots/Datum/04_Tag/01_sw-arqy/0010_sw-arqy_02.png</v>
       </c>
     </row>
@@ -24258,7 +24344,7 @@
         <v>1092</v>
       </c>
       <c r="L367" s="57" t="str">
-        <f t="shared" si="55"/>
+        <f t="shared" si="56"/>
         <v>02_Slots/Datum/04_Tag/01_sw-arqy/0020_sw-arqy_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -24291,7 +24377,7 @@
         <v>1092</v>
       </c>
       <c r="L368" s="57" t="str">
-        <f t="shared" si="55"/>
+        <f t="shared" si="56"/>
         <v>02_Slots/Datum/04_Tag/01_sw-arqy/0030_sw-arqy_NR_02.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -24563,7 +24649,7 @@
         <v>111</v>
       </c>
       <c r="L384" s="57" t="str">
-        <f t="shared" ref="L384" si="56">_xlfn.TEXTJOIN("", TRUE, D384:J384)</f>
+        <f t="shared" ref="L384" si="57">_xlfn.TEXTJOIN("", TRUE, D384:J384)</f>
         <v>02_Slots/Datum/02_Monat/0010_tpy_01.png</v>
       </c>
     </row>
@@ -24657,7 +24743,7 @@
         <v>1408</v>
       </c>
       <c r="L390" s="57" t="str">
-        <f t="shared" ref="L390:L393" si="57">_xlfn.TEXTJOIN("", TRUE, D390:K390)</f>
+        <f t="shared" ref="L390:L393" si="58">_xlfn.TEXTJOIN("", TRUE, D390:K390)</f>
         <v>02_Slots/Datum/04_Tag/01_sw-arqy/0001_sw-arqy_01.png</v>
       </c>
     </row>
@@ -24681,7 +24767,7 @@
         <v>1409</v>
       </c>
       <c r="L391" s="57" t="str">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>02_Slots/Datum/04_Tag/01_sw-arqy/0010_sw-arqy_02.png</v>
       </c>
     </row>
@@ -24714,7 +24800,7 @@
         <v>1092</v>
       </c>
       <c r="L392" s="57" t="str">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>02_Slots/Datum/04_Tag/01_sw-arqy/0020_sw-arqy_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -24747,7 +24833,7 @@
         <v>1092</v>
       </c>
       <c r="L393" s="57" t="str">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>02_Slots/Datum/04_Tag/01_sw-arqy/0030_sw-arqy_NR_02.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -24856,7 +24942,7 @@
         <v>886</v>
       </c>
       <c r="L410" s="57" t="str">
-        <f t="shared" ref="L410" si="58">_xlfn.TEXTJOIN("", TRUE, D410:J410)</f>
+        <f t="shared" ref="L410" si="59">_xlfn.TEXTJOIN("", TRUE, D410:J410)</f>
         <v>02_Slots/Koenig/01_Horusname_01/0001_Hr_01.png</v>
       </c>
     </row>
@@ -24922,7 +25008,7 @@
         <v>1092</v>
       </c>
       <c r="L412" s="57" t="str">
-        <f t="shared" ref="L412:L415" si="59">_xlfn.TEXTJOIN("", TRUE, D412:K412)</f>
+        <f t="shared" ref="L412:L415" si="60">_xlfn.TEXTJOIN("", TRUE, D412:K412)</f>
         <v>02_Slots/Koenig/01_Horusname_01/0020_Hr_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -24955,7 +25041,7 @@
         <v>1092</v>
       </c>
       <c r="L413" s="57" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>02_Slots/Koenig/01_Horusname_01/0030_Hr_MR_02.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -24988,7 +25074,7 @@
         <v>1092</v>
       </c>
       <c r="L414" s="57" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>02_Slots/Koenig/01_Horusname_01/0040_Hr_D.19_01.png &lt;sup&gt;(D.19)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -25021,7 +25107,7 @@
         <v>1092</v>
       </c>
       <c r="L415" s="57" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>02_Slots/Koenig/01_Horusname_01/0050_Hr_D.19_02.png &lt;sup&gt;(D.19)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -25112,7 +25198,7 @@
         <v>1523</v>
       </c>
       <c r="L421" s="57" t="str">
-        <f t="shared" ref="L421" si="60">_xlfn.TEXTJOIN("", TRUE, D421:J421)</f>
+        <f t="shared" ref="L421" si="61">_xlfn.TEXTJOIN("", TRUE, D421:J421)</f>
         <v>02_Slots/Koenig/02_Herrinname_01/0001_nbty_01.png</v>
       </c>
     </row>
@@ -25145,7 +25231,7 @@
         <v>1092</v>
       </c>
       <c r="L422" s="57" t="str">
-        <f t="shared" ref="L422" si="61">_xlfn.TEXTJOIN("", TRUE, D422:K422)</f>
+        <f t="shared" ref="L422" si="62">_xlfn.TEXTJOIN("", TRUE, D422:K422)</f>
         <v>02_Slots/Koenig/02_Herrinname_01/0010_nbty_Gr_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -25236,7 +25322,7 @@
         <v>1525</v>
       </c>
       <c r="L428" s="57" t="str">
-        <f t="shared" ref="L428" si="62">_xlfn.TEXTJOIN("", TRUE, D428:K428)</f>
+        <f t="shared" ref="L428" si="63">_xlfn.TEXTJOIN("", TRUE, D428:K428)</f>
         <v>02_Slots/Koenig/03_Goldhorus_01/0001_Hr-m-nb.w_01.png</v>
       </c>
     </row>
@@ -25330,7 +25416,7 @@
         <v>1526</v>
       </c>
       <c r="L434" s="57" t="str">
-        <f t="shared" ref="L434:L438" si="63">_xlfn.TEXTJOIN("", TRUE, D434:K434)</f>
+        <f t="shared" ref="L434:L438" si="64">_xlfn.TEXTJOIN("", TRUE, D434:K434)</f>
         <v>02_Slots/Koenig/04_Thronname_01/0001_nsw-bit_01.png</v>
       </c>
     </row>
@@ -25354,7 +25440,7 @@
         <v>1527</v>
       </c>
       <c r="L435" s="57" t="str">
-        <f t="shared" si="63"/>
+        <f t="shared" si="64"/>
         <v>02_Slots/Koenig/04_Thronname_01/0010_nsw-bit_02.png</v>
       </c>
     </row>
@@ -25387,7 +25473,7 @@
         <v>1092</v>
       </c>
       <c r="L436" s="57" t="str">
-        <f t="shared" si="63"/>
+        <f t="shared" si="64"/>
         <v>02_Slots/Koenig/04_Thronname_01/0020_nsw-bit_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -25420,7 +25506,7 @@
         <v>1092</v>
       </c>
       <c r="L437" s="57" t="str">
-        <f t="shared" si="63"/>
+        <f t="shared" si="64"/>
         <v>02_Slots/Koenig/04_Thronname_01/0030_nsw-bit_NR_02.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -25453,7 +25539,7 @@
         <v>1092</v>
       </c>
       <c r="L438" s="57" t="str">
-        <f t="shared" si="63"/>
+        <f t="shared" si="64"/>
         <v>02_Slots/Koenig/04_Thronname_01/0040_nsw-bit_NR_03.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -25486,7 +25572,7 @@
         <v>1092</v>
       </c>
       <c r="L439" s="57" t="str">
-        <f t="shared" ref="L439" si="64">_xlfn.TEXTJOIN("", TRUE, D439:K439)</f>
+        <f t="shared" ref="L439" si="65">_xlfn.TEXTJOIN("", TRUE, D439:K439)</f>
         <v>02_Slots/Koenig/04_Thronname_01/0050_nsw-bit_NR_04.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -25519,7 +25605,7 @@
         <v>1092</v>
       </c>
       <c r="L440" s="57" t="str">
-        <f t="shared" ref="L440:L441" si="65">_xlfn.TEXTJOIN("", TRUE, D440:K440)</f>
+        <f t="shared" ref="L440:L441" si="66">_xlfn.TEXTJOIN("", TRUE, D440:K440)</f>
         <v>02_Slots/Koenig/04_Thronname_01/0060_nsw-bit_Gr_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -25552,7 +25638,7 @@
         <v>1092</v>
       </c>
       <c r="L441" s="57" t="str">
-        <f t="shared" si="65"/>
+        <f t="shared" si="66"/>
         <v>02_Slots/Koenig/04_Thronname_01/0070_nsw-bit_Gr_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -25585,7 +25671,7 @@
         <v>1092</v>
       </c>
       <c r="L442" s="57" t="str">
-        <f t="shared" ref="L442:L443" si="66">_xlfn.TEXTJOIN("", TRUE, D442:K442)</f>
+        <f t="shared" ref="L442:L443" si="67">_xlfn.TEXTJOIN("", TRUE, D442:K442)</f>
         <v>02_Slots/Koenig/04_Thronname_01/0080_nsw-bit_Gr_03.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -25618,7 +25704,7 @@
         <v>1092</v>
       </c>
       <c r="L443" s="57" t="str">
-        <f t="shared" si="66"/>
+        <f t="shared" si="67"/>
         <v>02_Slots/Koenig/04_Thronname_01/0090_nsw-bit_Gr_04.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -25709,7 +25795,7 @@
         <v>1536</v>
       </c>
       <c r="L449" s="57" t="str">
-        <f t="shared" ref="L449:L450" si="67">_xlfn.TEXTJOIN("", TRUE, D449:K449)</f>
+        <f t="shared" ref="L449:L450" si="68">_xlfn.TEXTJOIN("", TRUE, D449:K449)</f>
         <v>02_Slots/Koenig/05_Eigenname_01/0001_sA-ra_01.png</v>
       </c>
     </row>
@@ -25742,7 +25828,7 @@
         <v>1092</v>
       </c>
       <c r="L450" s="57" t="str">
-        <f t="shared" si="67"/>
+        <f t="shared" si="68"/>
         <v>02_Slots/Koenig/05_Eigenname_01/0010_sA-ra_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -25775,7 +25861,7 @@
         <v>1092</v>
       </c>
       <c r="L451" s="57" t="str">
-        <f t="shared" ref="L451:L452" si="68">_xlfn.TEXTJOIN("", TRUE, D451:K451)</f>
+        <f t="shared" ref="L451:L452" si="69">_xlfn.TEXTJOIN("", TRUE, D451:K451)</f>
         <v>02_Slots/Koenig/05_Eigenname_01/0020_sA-ra_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -25808,7 +25894,7 @@
         <v>1092</v>
       </c>
       <c r="L452" s="57" t="str">
-        <f t="shared" si="68"/>
+        <f t="shared" si="69"/>
         <v>02_Slots/Koenig/05_Eigenname_01/0030_sA-ra_D.20_01.png &lt;sup&gt;(D.20)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -25841,7 +25927,7 @@
         <v>1092</v>
       </c>
       <c r="L453" s="57" t="str">
-        <f t="shared" ref="L453:L454" si="69">_xlfn.TEXTJOIN("", TRUE, D453:K453)</f>
+        <f t="shared" ref="L453:L454" si="70">_xlfn.TEXTJOIN("", TRUE, D453:K453)</f>
         <v>02_Slots/Koenig/05_Eigenname_01/0040_sA-ra_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -25874,7 +25960,7 @@
         <v>1092</v>
       </c>
       <c r="L454" s="57" t="str">
-        <f t="shared" si="69"/>
+        <f t="shared" si="70"/>
         <v>02_Slots/Koenig/05_Eigenname_01/0050_sA-ra_Gr_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -25965,7 +26051,7 @@
         <v>1303</v>
       </c>
       <c r="L461" s="57" t="str">
-        <f t="shared" ref="L461:L463" si="70">_xlfn.TEXTJOIN("", TRUE, D461:J461)</f>
+        <f t="shared" ref="L461:L463" si="71">_xlfn.TEXTJOIN("", TRUE, D461:J461)</f>
         <v>02_Slots/Koenig/Epitheta/06_nsw/0001_nsw_01.png</v>
       </c>
     </row>
@@ -25989,7 +26075,7 @@
         <v>1304</v>
       </c>
       <c r="L462" s="57" t="str">
-        <f t="shared" si="70"/>
+        <f t="shared" si="71"/>
         <v>02_Slots/Koenig/Epitheta/06_nsw/0010_nsw_02.png</v>
       </c>
     </row>
@@ -26013,7 +26099,7 @@
         <v>1305</v>
       </c>
       <c r="L463" s="57" t="str">
-        <f t="shared" si="70"/>
+        <f t="shared" si="71"/>
         <v>02_Slots/Koenig/Epitheta/06_nsw/0020_nsw_03.png</v>
       </c>
     </row>
@@ -26079,7 +26165,7 @@
         <v>1297</v>
       </c>
       <c r="L468" s="57" t="str">
-        <f t="shared" ref="L468:L470" si="71">_xlfn.TEXTJOIN("", TRUE, D468:J468)</f>
+        <f t="shared" ref="L468:L470" si="72">_xlfn.TEXTJOIN("", TRUE, D468:J468)</f>
         <v>02_Slots/Koenig/Epitheta/05_Hm/0001_Hm_01.png</v>
       </c>
     </row>
@@ -26103,7 +26189,7 @@
         <v>1298</v>
       </c>
       <c r="L469" s="57" t="str">
-        <f t="shared" si="71"/>
+        <f t="shared" si="72"/>
         <v>02_Slots/Koenig/Epitheta/05_Hm/0010_Hm_02.png</v>
       </c>
     </row>
@@ -26127,7 +26213,7 @@
         <v>1299</v>
       </c>
       <c r="L470" s="57" t="str">
-        <f t="shared" si="71"/>
+        <f t="shared" si="72"/>
         <v>02_Slots/Koenig/Epitheta/05_Hm/0020_Hm_03.png</v>
       </c>
     </row>
@@ -26196,7 +26282,7 @@
         <v>111</v>
       </c>
       <c r="L475" s="57" t="str">
-        <f t="shared" ref="L475" si="72">_xlfn.TEXTJOIN("", TRUE, D475:J475)</f>
+        <f t="shared" ref="L475" si="73">_xlfn.TEXTJOIN("", TRUE, D475:J475)</f>
         <v>02_Slots/Koenig/Epitheta/04_Hm=f/0001_Hm=f_01.png</v>
       </c>
     </row>
@@ -26265,7 +26351,7 @@
         <v>111</v>
       </c>
       <c r="L480" s="57" t="str">
-        <f t="shared" ref="L480" si="73">_xlfn.TEXTJOIN("", TRUE, D480:J480)</f>
+        <f t="shared" ref="L480" si="74">_xlfn.TEXTJOIN("", TRUE, D480:J480)</f>
         <v>02_Slots/Koenig/Epitheta/02_nb-tA.wj/0001_nb-tA.wj_01.png</v>
       </c>
     </row>
@@ -26334,7 +26420,7 @@
         <v>111</v>
       </c>
       <c r="L485" s="57" t="str">
-        <f t="shared" ref="L485" si="74">_xlfn.TEXTJOIN("", TRUE, D485:J485)</f>
+        <f t="shared" ref="L485" si="75">_xlfn.TEXTJOIN("", TRUE, D485:J485)</f>
         <v>02_Slots/Koenig/Epitheta/01_nTr-nfr/0001_nTr-nfr_01.png</v>
       </c>
     </row>
@@ -26689,7 +26775,7 @@
         <v>111</v>
       </c>
       <c r="L516" s="57" t="str">
-        <f t="shared" ref="L516:L522" si="75">_xlfn.TEXTJOIN("", TRUE, D516:J516)</f>
+        <f t="shared" ref="L516:L522" si="76">_xlfn.TEXTJOIN("", TRUE, D516:J516)</f>
         <v>02_Slots/Gottheit/Determinative_typisch/01_m/0001_A40_01.png</v>
       </c>
     </row>
@@ -26713,7 +26799,7 @@
         <v>111</v>
       </c>
       <c r="L517" s="57" t="str">
-        <f t="shared" si="75"/>
+        <f t="shared" si="76"/>
         <v>02_Slots/Gottheit/Determinative_typisch/01_m/0010_G7_01.png</v>
       </c>
     </row>
@@ -26737,7 +26823,7 @@
         <v>111</v>
       </c>
       <c r="L518" s="57" t="str">
-        <f t="shared" si="75"/>
+        <f t="shared" si="76"/>
         <v>02_Slots/Gottheit/Determinative_typisch/01_m/0020_R8_01.png</v>
       </c>
     </row>
@@ -26761,7 +26847,7 @@
         <v>111</v>
       </c>
       <c r="L519" s="57" t="str">
-        <f t="shared" si="75"/>
+        <f t="shared" si="76"/>
         <v>02_Slots/Gottheit/Determinative_typisch/02_f/0001_B7_01.png</v>
       </c>
     </row>
@@ -26785,7 +26871,7 @@
         <v>111</v>
       </c>
       <c r="L520" s="57" t="str">
-        <f t="shared" si="75"/>
+        <f t="shared" si="76"/>
         <v>02_Slots/Gottheit/Determinative_typisch/02_f/0010_I64_01.png</v>
       </c>
     </row>
@@ -26809,7 +26895,7 @@
         <v>111</v>
       </c>
       <c r="L521" s="57" t="str">
-        <f t="shared" si="75"/>
+        <f t="shared" si="76"/>
         <v>02_Slots/Gottheit/Determinative_typisch/02_f/0020_H8_01.png</v>
       </c>
     </row>
@@ -26833,7 +26919,7 @@
         <v>111</v>
       </c>
       <c r="L522" s="57" t="str">
-        <f t="shared" si="75"/>
+        <f t="shared" si="76"/>
         <v>02_Slots/Gottheit/Determinative_typisch/02_f/0030_H8_02.png</v>
       </c>
     </row>
@@ -26868,7 +26954,7 @@
         <v>947</v>
       </c>
       <c r="L525" s="57" t="str">
-        <f t="shared" ref="L525" si="76">_xlfn.TEXTJOIN("", TRUE, D525:J525)</f>
+        <f t="shared" ref="L525" si="77">_xlfn.TEXTJOIN("", TRUE, D525:J525)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0010_Isis/0001_st_01.png</v>
       </c>
     </row>
@@ -26898,7 +26984,7 @@
         <v>1092</v>
       </c>
       <c r="L526" s="57" t="str">
-        <f t="shared" ref="L526:L529" si="77">_xlfn.TEXTJOIN("", TRUE, D526:K526)</f>
+        <f t="shared" ref="L526:L529" si="78">_xlfn.TEXTJOIN("", TRUE, D526:K526)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0010_Isis/0010_st_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -26928,7 +27014,7 @@
         <v>1092</v>
       </c>
       <c r="L527" s="57" t="str">
-        <f t="shared" si="77"/>
+        <f t="shared" si="78"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0010_Isis/0020_st_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -26958,7 +27044,7 @@
         <v>1092</v>
       </c>
       <c r="L528" s="57" t="str">
-        <f t="shared" si="77"/>
+        <f t="shared" si="78"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0010_Isis/0030_st_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -26988,7 +27074,7 @@
         <v>1092</v>
       </c>
       <c r="L529" s="57" t="str">
-        <f t="shared" si="77"/>
+        <f t="shared" si="78"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0010_Isis/0040_st_SP_01.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -27003,7 +27089,7 @@
         <v>105</v>
       </c>
       <c r="L530" s="57" t="str">
-        <f t="shared" ref="L530" si="78">_xlfn.TEXTJOIN("", TRUE, D530:J530)</f>
+        <f t="shared" ref="L530" si="79">_xlfn.TEXTJOIN("", TRUE, D530:J530)</f>
         <v/>
       </c>
     </row>
@@ -27338,7 +27424,7 @@
         <v>1092</v>
       </c>
       <c r="L554" s="57" t="str">
-        <f t="shared" ref="L554:L555" si="79">_xlfn.TEXTJOIN("", TRUE, D554:K554)</f>
+        <f t="shared" ref="L554:L555" si="80">_xlfn.TEXTJOIN("", TRUE, D554:K554)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0020_Amun/0010_Jmn_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -27371,7 +27457,7 @@
         <v>1092</v>
       </c>
       <c r="L555" s="57" t="str">
-        <f t="shared" si="79"/>
+        <f t="shared" si="80"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0020_Amun/0020_Jmn_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -27481,7 +27567,7 @@
         <v>111</v>
       </c>
       <c r="L562" s="57" t="str">
-        <f t="shared" ref="L562:L563" si="80">_xlfn.TEXTJOIN("", TRUE, D562:K562)</f>
+        <f t="shared" ref="L562:L563" si="81">_xlfn.TEXTJOIN("", TRUE, D562:K562)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0020_Amun/epitheta/01_m-jp.t/0010_m-jp.t_01.png</v>
       </c>
     </row>
@@ -27517,7 +27603,7 @@
         <v>1092</v>
       </c>
       <c r="L563" s="57" t="str">
-        <f t="shared" si="80"/>
+        <f t="shared" si="81"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0020_Amun/epitheta/01_m-jp.t/0020_m-jp.t_SP_01.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -27768,7 +27854,7 @@
         <v>111</v>
       </c>
       <c r="L582" s="57" t="str">
-        <f t="shared" ref="L582:L584" si="81">_xlfn.TEXTJOIN("", TRUE, D582:J582)</f>
+        <f t="shared" ref="L582:L584" si="82">_xlfn.TEXTJOIN("", TRUE, D582:J582)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0050_Amset/0001_jmstj_01.png</v>
       </c>
     </row>
@@ -27792,7 +27878,7 @@
         <v>111</v>
       </c>
       <c r="L583" s="57" t="str">
-        <f t="shared" si="81"/>
+        <f t="shared" si="82"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0050_Amset/0010_jmstj_02.png</v>
       </c>
     </row>
@@ -27816,7 +27902,7 @@
         <v>111</v>
       </c>
       <c r="L584" s="57" t="str">
-        <f t="shared" si="81"/>
+        <f t="shared" si="82"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0050_Amset/0020_jmstj_03.png</v>
       </c>
     </row>
@@ -27849,7 +27935,7 @@
         <v>1092</v>
       </c>
       <c r="L585" s="57" t="str">
-        <f t="shared" ref="L585:L588" si="82">_xlfn.TEXTJOIN("", TRUE, D585:K585)</f>
+        <f t="shared" ref="L585:L588" si="83">_xlfn.TEXTJOIN("", TRUE, D585:K585)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0050_Amset/0030_jmstj_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -27882,7 +27968,7 @@
         <v>1092</v>
       </c>
       <c r="L586" s="57" t="str">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0050_Amset/0040_jmstj_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -27915,7 +28001,7 @@
         <v>1092</v>
       </c>
       <c r="L587" s="57" t="str">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0050_Amset/0050_jmstj_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -27948,7 +28034,7 @@
         <v>1092</v>
       </c>
       <c r="L588" s="57" t="str">
-        <f t="shared" si="82"/>
+        <f t="shared" si="83"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0050_Amset/0060_jmstj_NR_02.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -28045,7 +28131,7 @@
         <v>111</v>
       </c>
       <c r="L597" s="57" t="str">
-        <f t="shared" ref="L597:L601" si="83">_xlfn.TEXTJOIN("", TRUE, D597:J597)</f>
+        <f t="shared" ref="L597:L601" si="84">_xlfn.TEXTJOIN("", TRUE, D597:J597)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0060_Onuris/0001_jnj-Hr.t_01.png</v>
       </c>
     </row>
@@ -28069,7 +28155,7 @@
         <v>111</v>
       </c>
       <c r="L598" s="57" t="str">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0060_Onuris/0010_jnj-Hr.t_02.png</v>
       </c>
     </row>
@@ -28093,7 +28179,7 @@
         <v>111</v>
       </c>
       <c r="L599" s="57" t="str">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0060_Onuris/0020_jnj-Hr.t_03.png</v>
       </c>
     </row>
@@ -28117,7 +28203,7 @@
         <v>111</v>
       </c>
       <c r="L600" s="57" t="str">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0060_Onuris/0030_jnj-Hr.t_04.png</v>
       </c>
     </row>
@@ -28141,7 +28227,7 @@
         <v>111</v>
       </c>
       <c r="L601" s="57" t="str">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0060_Onuris/0040_jnj-Hr.t_05.png</v>
       </c>
     </row>
@@ -28268,7 +28354,7 @@
         <v>111</v>
       </c>
       <c r="L610" s="57" t="str">
-        <f t="shared" ref="L610:L615" si="84">_xlfn.TEXTJOIN("", TRUE, D610:J610)</f>
+        <f t="shared" ref="L610:L615" si="85">_xlfn.TEXTJOIN("", TRUE, D610:J610)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0070_Anubis/0001_Jnpw_01.png</v>
       </c>
     </row>
@@ -28292,7 +28378,7 @@
         <v>111</v>
       </c>
       <c r="L611" s="57" t="str">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0070_Anubis/0010_Jnpw_02.png</v>
       </c>
     </row>
@@ -28316,7 +28402,7 @@
         <v>111</v>
       </c>
       <c r="L612" s="57" t="str">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0070_Anubis/0020_Jnpw_03.png</v>
       </c>
     </row>
@@ -28340,7 +28426,7 @@
         <v>111</v>
       </c>
       <c r="L613" s="57" t="str">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0070_Anubis/0030_Jnpw_04.png</v>
       </c>
     </row>
@@ -28400,7 +28486,7 @@
         <v>111</v>
       </c>
       <c r="L615" s="57" t="str">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0070_Anubis/det/0001_Jnpw_det_01.png</v>
       </c>
     </row>
@@ -28546,7 +28632,7 @@
         <v>1092</v>
       </c>
       <c r="L623" s="57" t="str">
-        <f t="shared" ref="L623:L624" si="85">_xlfn.TEXTJOIN("", TRUE, D623:K623)</f>
+        <f t="shared" ref="L623:L624" si="86">_xlfn.TEXTJOIN("", TRUE, D623:K623)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0070_Anubis/epitheta/01_jmj-wt/0020_jmj-wt_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -28582,7 +28668,7 @@
         <v>1092</v>
       </c>
       <c r="L624" s="57" t="str">
-        <f t="shared" si="85"/>
+        <f t="shared" si="86"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0070_Anubis/epitheta/01_jmj-wt/0030_jmj-wt_AR_02.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -28888,7 +28974,7 @@
         <v>1092</v>
       </c>
       <c r="L642" s="57" t="str">
-        <f t="shared" ref="L642:L650" si="86">_xlfn.TEXTJOIN("", TRUE, D642:K642)</f>
+        <f t="shared" ref="L642:L650" si="87">_xlfn.TEXTJOIN("", TRUE, D642:K642)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0070_Anubis/epitheta/04_xnt.j-sH-nTr/0001_xnt.j-sH-nTr_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -28924,7 +29010,7 @@
         <v>1092</v>
       </c>
       <c r="L643" s="57" t="str">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0070_Anubis/epitheta/04_xnt.j-sH-nTr/0010_xnt.j-sH-nTr_AR_02.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -28960,7 +29046,7 @@
         <v>1092</v>
       </c>
       <c r="L644" s="57" t="str">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0070_Anubis/epitheta/04_xnt.j-sH-nTr/0020_xnt.j-sH-nTr_AR_03.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -28996,7 +29082,7 @@
         <v>1092</v>
       </c>
       <c r="L645" s="57" t="str">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0070_Anubis/epitheta/04_xnt.j-sH-nTr/0030_xnt.j-sH-nTr_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -29032,7 +29118,7 @@
         <v>1092</v>
       </c>
       <c r="L646" s="57" t="str">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0070_Anubis/epitheta/04_xnt.j-sH-nTr/0040_xnt.j-sH-nTr_MR_02.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -29068,7 +29154,7 @@
         <v>1092</v>
       </c>
       <c r="L647" s="57" t="str">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0070_Anubis/epitheta/04_xnt.j-sH-nTr/0050_xnt.j-sH-nTr_D.18_01.png &lt;sup&gt;(D.18)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -29104,7 +29190,7 @@
         <v>1092</v>
       </c>
       <c r="L648" s="57" t="str">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0070_Anubis/epitheta/04_xnt.j-sH-nTr/0060_xnt.j-sH-nTr_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -29140,7 +29226,7 @@
         <v>1092</v>
       </c>
       <c r="L649" s="57" t="str">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0070_Anubis/epitheta/04_xnt.j-sH-nTr/0070_xnt.j-sH-nTr_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -29176,7 +29262,7 @@
         <v>1092</v>
       </c>
       <c r="L650" s="57" t="str">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0070_Anubis/epitheta/04_xnt.j-sH-nTr/0080_xnt.j-sH-nTr_GR_03.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -29242,7 +29328,7 @@
         <v>111</v>
       </c>
       <c r="L659" s="57" t="str">
-        <f t="shared" ref="L659:L661" si="87">_xlfn.TEXTJOIN("", TRUE, D659:J659)</f>
+        <f t="shared" ref="L659:L661" si="88">_xlfn.TEXTJOIN("", TRUE, D659:J659)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0080_Atum/0001_Jtm_01.png</v>
       </c>
     </row>
@@ -29266,7 +29352,7 @@
         <v>111</v>
       </c>
       <c r="L660" s="57" t="str">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0080_Atum/0010_Jtm_02.png</v>
       </c>
     </row>
@@ -29290,7 +29376,7 @@
         <v>111</v>
       </c>
       <c r="L661" s="57" t="str">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0080_Atum/0020_Jtm_03.png</v>
       </c>
     </row>
@@ -29323,7 +29409,7 @@
         <v>1092</v>
       </c>
       <c r="L662" s="57" t="str">
-        <f t="shared" ref="L662:L665" si="88">_xlfn.TEXTJOIN("", TRUE, D662:K662)</f>
+        <f t="shared" ref="L662:L665" si="89">_xlfn.TEXTJOIN("", TRUE, D662:K662)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0080_Atum/0030_Jtm_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -29356,7 +29442,7 @@
         <v>1092</v>
       </c>
       <c r="L663" s="57" t="str">
-        <f t="shared" si="88"/>
+        <f t="shared" si="89"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0080_Atum/0040_Jtm_MR_02.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -29389,7 +29475,7 @@
         <v>1092</v>
       </c>
       <c r="L664" s="57" t="str">
-        <f t="shared" si="88"/>
+        <f t="shared" si="89"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0080_Atum/0050_Jtm_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -29422,7 +29508,7 @@
         <v>1092</v>
       </c>
       <c r="L665" s="57" t="str">
-        <f t="shared" si="88"/>
+        <f t="shared" si="89"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0080_Atum/0060_Jtm_SP_01.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -29666,7 +29752,7 @@
         <v>1092</v>
       </c>
       <c r="L681" s="57" t="str">
-        <f t="shared" ref="L681:L683" si="89">_xlfn.TEXTJOIN("", TRUE, D681:K681)</f>
+        <f t="shared" ref="L681:L683" si="90">_xlfn.TEXTJOIN("", TRUE, D681:K681)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0090_Aton/0020_jtn_D.18_01.png &lt;sup&gt;(D.18)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -29699,7 +29785,7 @@
         <v>1092</v>
       </c>
       <c r="L682" s="57" t="str">
-        <f t="shared" si="89"/>
+        <f t="shared" si="90"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0090_Aton/0030_jtn_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -29732,7 +29818,7 @@
         <v>1092</v>
       </c>
       <c r="L683" s="57" t="str">
-        <f t="shared" si="89"/>
+        <f t="shared" si="90"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0090_Aton/0040_jtn_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -30272,7 +30358,7 @@
         <v>111</v>
       </c>
       <c r="L722" s="57" t="str">
-        <f t="shared" ref="L722:L732" si="90">_xlfn.TEXTJOIN("", TRUE, D722:J722)</f>
+        <f t="shared" ref="L722:L732" si="91">_xlfn.TEXTJOIN("", TRUE, D722:J722)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/0001_wsjr_01.png</v>
       </c>
     </row>
@@ -30296,7 +30382,7 @@
         <v>111</v>
       </c>
       <c r="L723" s="57" t="str">
-        <f t="shared" si="90"/>
+        <f t="shared" si="91"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/0010_wsjr_02.png</v>
       </c>
     </row>
@@ -30320,7 +30406,7 @@
         <v>111</v>
       </c>
       <c r="L724" s="57" t="str">
-        <f t="shared" si="90"/>
+        <f t="shared" si="91"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/0020_wsjr_03.png</v>
       </c>
     </row>
@@ -30353,7 +30439,7 @@
         <v>1092</v>
       </c>
       <c r="L725" s="57" t="str">
-        <f t="shared" ref="L725:L731" si="91">_xlfn.TEXTJOIN("", TRUE, D725:K725)</f>
+        <f t="shared" ref="L725:L731" si="92">_xlfn.TEXTJOIN("", TRUE, D725:K725)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/0030_wsjr_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -30386,7 +30472,7 @@
         <v>1092</v>
       </c>
       <c r="L726" s="57" t="str">
-        <f t="shared" si="91"/>
+        <f t="shared" si="92"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/0040_wsjr_MR_02.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -30419,7 +30505,7 @@
         <v>1092</v>
       </c>
       <c r="L727" s="57" t="str">
-        <f t="shared" si="91"/>
+        <f t="shared" si="92"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/0050_wsjr_MR_03.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -30452,7 +30538,7 @@
         <v>1092</v>
       </c>
       <c r="L728" s="57" t="str">
-        <f t="shared" si="91"/>
+        <f t="shared" si="92"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/0060_wsjr_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -30485,7 +30571,7 @@
         <v>1092</v>
       </c>
       <c r="L729" s="57" t="str">
-        <f t="shared" si="91"/>
+        <f t="shared" si="92"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/0070_wsjr_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -30518,7 +30604,7 @@
         <v>1092</v>
       </c>
       <c r="L730" s="57" t="str">
-        <f t="shared" si="91"/>
+        <f t="shared" si="92"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/0080_wsjr_GR_03.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -30551,7 +30637,7 @@
         <v>1092</v>
       </c>
       <c r="L731" s="57" t="str">
-        <f t="shared" si="91"/>
+        <f t="shared" si="92"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/0090_wsjr_GR_04.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -30578,7 +30664,7 @@
         <v>111</v>
       </c>
       <c r="L732" s="57" t="str">
-        <f t="shared" si="90"/>
+        <f t="shared" si="91"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/det/0001_wsjr_det_01.png</v>
       </c>
     </row>
@@ -30751,7 +30837,7 @@
         <v>1092</v>
       </c>
       <c r="L741" s="57" t="str">
-        <f t="shared" ref="L741:L742" si="92">_xlfn.TEXTJOIN("", TRUE, D741:K741)</f>
+        <f t="shared" ref="L741:L742" si="93">_xlfn.TEXTJOIN("", TRUE, D741:K741)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/epitheta/01_nb-AbDw/0030_nb-AbDw_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -30787,7 +30873,7 @@
         <v>1092</v>
       </c>
       <c r="L742" s="57" t="str">
-        <f t="shared" si="92"/>
+        <f t="shared" si="93"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/epitheta/01_nb-AbDw/0040_nb-AbDw_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -30856,7 +30942,7 @@
         <v>111</v>
       </c>
       <c r="L747" s="57" t="str">
-        <f t="shared" ref="L747:L754" si="93">_xlfn.TEXTJOIN("", TRUE, D747:J747)</f>
+        <f t="shared" ref="L747:L754" si="94">_xlfn.TEXTJOIN("", TRUE, D747:J747)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/epitheta/02_nb-Dd.w/0001_nb-Dd.w_01.png</v>
       </c>
     </row>
@@ -30880,7 +30966,7 @@
         <v>693</v>
       </c>
       <c r="L748" s="57" t="str">
-        <f t="shared" si="93"/>
+        <f t="shared" si="94"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/epitheta/02_nb-Dd.w/0010_nb-Dd.w_02.png</v>
       </c>
     </row>
@@ -30904,7 +30990,7 @@
         <v>694</v>
       </c>
       <c r="L749" s="57" t="str">
-        <f t="shared" si="93"/>
+        <f t="shared" si="94"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/epitheta/02_nb-Dd.w/0020_nb-Dd.w_03.png</v>
       </c>
     </row>
@@ -30928,7 +31014,7 @@
         <v>695</v>
       </c>
       <c r="L750" s="57" t="str">
-        <f t="shared" si="93"/>
+        <f t="shared" si="94"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/epitheta/02_nb-Dd.w/0030_nb-Dd.w_04.png</v>
       </c>
     </row>
@@ -30952,7 +31038,7 @@
         <v>696</v>
       </c>
       <c r="L751" s="57" t="str">
-        <f t="shared" si="93"/>
+        <f t="shared" si="94"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/epitheta/02_nb-Dd.w/0040_nb-Dd.w_05.png</v>
       </c>
     </row>
@@ -30976,7 +31062,7 @@
         <v>697</v>
       </c>
       <c r="L752" s="57" t="str">
-        <f t="shared" si="93"/>
+        <f t="shared" si="94"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/epitheta/02_nb-Dd.w/0050_nb-Dd.w_06.png</v>
       </c>
     </row>
@@ -31000,7 +31086,7 @@
         <v>698</v>
       </c>
       <c r="L753" s="57" t="str">
-        <f t="shared" si="93"/>
+        <f t="shared" si="94"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/epitheta/02_nb-Dd.w/0060_nb-Dd.w_07.png</v>
       </c>
     </row>
@@ -31024,7 +31110,7 @@
         <v>699</v>
       </c>
       <c r="L754" s="57" t="str">
-        <f t="shared" si="93"/>
+        <f t="shared" si="94"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/epitheta/02_nb-Dd.w/0070_nb-Dd.w_08.png</v>
       </c>
     </row>
@@ -31258,7 +31344,7 @@
         <v>703</v>
       </c>
       <c r="L770" s="57" t="str">
-        <f t="shared" ref="L770:L771" si="94">_xlfn.TEXTJOIN("", TRUE, D770:J770)</f>
+        <f t="shared" ref="L770:L771" si="95">_xlfn.TEXTJOIN("", TRUE, D770:J770)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/epitheta/05_xnt.y-jmn.ty.w/0001_xnt.y-jmn.ty.w_01.png</v>
       </c>
     </row>
@@ -31282,7 +31368,7 @@
         <v>704</v>
       </c>
       <c r="L771" s="57" t="str">
-        <f t="shared" si="94"/>
+        <f t="shared" si="95"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/epitheta/05_xnt.y-jmn.ty.w/0010_xnt.y-jmn.ty.w_02.png</v>
       </c>
     </row>
@@ -31315,7 +31401,7 @@
         <v>1092</v>
       </c>
       <c r="L772" s="57" t="str">
-        <f t="shared" ref="L772:L776" si="95">_xlfn.TEXTJOIN("", TRUE, D772:K772)</f>
+        <f t="shared" ref="L772:L776" si="96">_xlfn.TEXTJOIN("", TRUE, D772:K772)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/epitheta/05_xnt.y-jmn.ty.w/0020_xnt.y-jmn.ty.w_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -31348,7 +31434,7 @@
         <v>1092</v>
       </c>
       <c r="L773" s="57" t="str">
-        <f t="shared" si="95"/>
+        <f t="shared" si="96"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/epitheta/05_xnt.y-jmn.ty.w/0030_xnt.y-jmn.ty.w_AR_02.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -31381,7 +31467,7 @@
         <v>1092</v>
       </c>
       <c r="L774" s="57" t="str">
-        <f t="shared" si="95"/>
+        <f t="shared" si="96"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/epitheta/05_xnt.y-jmn.ty.w/0040_xnt.y-jmn.ty.w_Pyr._01.png &lt;sup&gt;(Pyr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -31414,7 +31500,7 @@
         <v>1092</v>
       </c>
       <c r="L775" s="57" t="str">
-        <f t="shared" si="95"/>
+        <f t="shared" si="96"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/epitheta/05_xnt.y-jmn.ty.w/0050_xnt.y-jmn.ty.w_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -31447,7 +31533,7 @@
         <v>1092</v>
       </c>
       <c r="L776" s="57" t="str">
-        <f t="shared" si="95"/>
+        <f t="shared" si="96"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0110_Osiris/epitheta/05_xnt.y-jmn.ty.w/0060_xnt.y-jmn.ty.w_typ.-ab-NR_01.png &lt;sup&gt;(ab NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -31713,7 +31799,7 @@
         <v>1092</v>
       </c>
       <c r="L798" s="57" t="str">
-        <f t="shared" ref="L798:L799" si="96">_xlfn.TEXTJOIN("", TRUE, D798:K798)</f>
+        <f t="shared" ref="L798:L799" si="97">_xlfn.TEXTJOIN("", TRUE, D798:K798)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0120_Bastet/0010_bAst.t_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -31743,7 +31829,7 @@
         <v>1092</v>
       </c>
       <c r="L799" s="57" t="str">
-        <f t="shared" si="96"/>
+        <f t="shared" si="97"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0120_Bastet/0020_bAst.t_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -31879,7 +31965,7 @@
         <v>1092</v>
       </c>
       <c r="L809" s="57" t="str">
-        <f t="shared" ref="L809:L810" si="97">_xlfn.TEXTJOIN("", TRUE, D809:K809)</f>
+        <f t="shared" ref="L809:L810" si="98">_xlfn.TEXTJOIN("", TRUE, D809:K809)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0130_Behedeti/0020_bHd.t_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -31909,7 +31995,7 @@
         <v>1092</v>
       </c>
       <c r="L810" s="57" t="str">
-        <f t="shared" si="97"/>
+        <f t="shared" si="98"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0130_Behedeti/0030_bHd.t_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -32172,7 +32258,7 @@
         <v>732</v>
       </c>
       <c r="L829" s="57" t="str">
-        <f t="shared" ref="L829" si="98">_xlfn.TEXTJOIN("", TRUE, D829:J829)</f>
+        <f t="shared" ref="L829" si="99">_xlfn.TEXTJOIN("", TRUE, D829:J829)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0140_Goetterneunheit/0001_psD.t_01.png</v>
       </c>
     </row>
@@ -32202,7 +32288,7 @@
         <v>1092</v>
       </c>
       <c r="L830" s="57" t="str">
-        <f t="shared" ref="L830:L840" si="99">_xlfn.TEXTJOIN("", TRUE, D830:K830)</f>
+        <f t="shared" ref="L830:L840" si="100">_xlfn.TEXTJOIN("", TRUE, D830:K830)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0140_Goetterneunheit/0010_psD.t_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -32232,7 +32318,7 @@
         <v>1092</v>
       </c>
       <c r="L831" s="57" t="str">
-        <f t="shared" si="99"/>
+        <f t="shared" si="100"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0140_Goetterneunheit/0020_psD.t_AR_02.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -32262,7 +32348,7 @@
         <v>1092</v>
       </c>
       <c r="L832" s="57" t="str">
-        <f t="shared" si="99"/>
+        <f t="shared" si="100"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0140_Goetterneunheit/0030_psD.t_AR_03.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -32292,7 +32378,7 @@
         <v>1092</v>
       </c>
       <c r="L833" s="57" t="str">
-        <f t="shared" si="99"/>
+        <f t="shared" si="100"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0140_Goetterneunheit/0040_psD.t_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -32322,7 +32408,7 @@
         <v>1092</v>
       </c>
       <c r="L834" s="57" t="str">
-        <f t="shared" si="99"/>
+        <f t="shared" si="100"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0140_Goetterneunheit/0050_psD.t_SP_01.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -32352,7 +32438,7 @@
         <v>1092</v>
       </c>
       <c r="L835" s="57" t="str">
-        <f t="shared" si="99"/>
+        <f t="shared" si="100"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0140_Goetterneunheit/0060_psD.t_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -32382,7 +32468,7 @@
         <v>1092</v>
       </c>
       <c r="L836" s="57" t="str">
-        <f t="shared" si="99"/>
+        <f t="shared" si="100"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0140_Goetterneunheit/0070_psD.t_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -32415,7 +32501,7 @@
         <v>1092</v>
       </c>
       <c r="L837" s="57" t="str">
-        <f t="shared" si="99"/>
+        <f t="shared" si="100"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0140_Goetterneunheit/det/0001_psD.t_det_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -32448,7 +32534,7 @@
         <v>1092</v>
       </c>
       <c r="L838" s="57" t="str">
-        <f t="shared" si="99"/>
+        <f t="shared" si="100"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0140_Goetterneunheit/det/0010_psD.t_det_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -32481,7 +32567,7 @@
         <v>1092</v>
       </c>
       <c r="L839" s="57" t="str">
-        <f t="shared" si="99"/>
+        <f t="shared" si="100"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0140_Goetterneunheit/det/0020_psD.t_det_MR_02.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -32514,7 +32600,7 @@
         <v>1092</v>
       </c>
       <c r="L840" s="57" t="str">
-        <f t="shared" si="99"/>
+        <f t="shared" si="100"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0140_Goetterneunheit/det/0030_psD.t_det_SP_01.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -32594,7 +32680,7 @@
         <v>750</v>
       </c>
       <c r="L846" s="57" t="str">
-        <f t="shared" ref="L846:L847" si="100">_xlfn.TEXTJOIN("", TRUE, D846:J846)</f>
+        <f t="shared" ref="L846:L847" si="101">_xlfn.TEXTJOIN("", TRUE, D846:J846)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0140_Goetterneunheit/epitheta/01_aA.t/0001_aA.t_01.png</v>
       </c>
     </row>
@@ -32618,7 +32704,7 @@
         <v>751</v>
       </c>
       <c r="L847" s="57" t="str">
-        <f t="shared" si="100"/>
+        <f t="shared" si="101"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0140_Goetterneunheit/epitheta/01_aA.t/0010_aA.t_02.png</v>
       </c>
     </row>
@@ -32651,7 +32737,7 @@
         <v>1092</v>
       </c>
       <c r="L848" s="57" t="str">
-        <f t="shared" ref="L848:L851" si="101">_xlfn.TEXTJOIN("", TRUE, D848:K848)</f>
+        <f t="shared" ref="L848:L851" si="102">_xlfn.TEXTJOIN("", TRUE, D848:K848)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0140_Goetterneunheit/epitheta/01_aA.t/0020_aA.t_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -32684,7 +32770,7 @@
         <v>1092</v>
       </c>
       <c r="L849" s="57" t="str">
-        <f t="shared" si="101"/>
+        <f t="shared" si="102"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0140_Goetterneunheit/epitheta/01_aA.t/0030_aA.t_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -32717,7 +32803,7 @@
         <v>1092</v>
       </c>
       <c r="L850" s="57" t="str">
-        <f t="shared" si="101"/>
+        <f t="shared" si="102"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0140_Goetterneunheit/epitheta/01_aA.t/0040_aA.t_MR_02.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -32750,7 +32836,7 @@
         <v>1092</v>
       </c>
       <c r="L851" s="57" t="str">
-        <f t="shared" si="101"/>
+        <f t="shared" si="102"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0140_Goetterneunheit/epitheta/01_aA.t/0050_aA.t_MR_03.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -32849,7 +32935,7 @@
         <v>1092</v>
       </c>
       <c r="L857" s="57" t="str">
-        <f t="shared" ref="L857:L860" si="102">_xlfn.TEXTJOIN("", TRUE, D857:K857)</f>
+        <f t="shared" ref="L857:L860" si="103">_xlfn.TEXTJOIN("", TRUE, D857:K857)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0140_Goetterneunheit/epitheta/02_nDs.t/0010_nDs.t_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -32882,7 +32968,7 @@
         <v>1092</v>
       </c>
       <c r="L858" s="57" t="str">
-        <f t="shared" si="102"/>
+        <f t="shared" si="103"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0140_Goetterneunheit/epitheta/02_nDs.t/0020_nDs.t_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -32915,7 +33001,7 @@
         <v>1092</v>
       </c>
       <c r="L859" s="57" t="str">
-        <f t="shared" si="102"/>
+        <f t="shared" si="103"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0140_Goetterneunheit/epitheta/02_nDs.t/0030_nDs.t_MR_02.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -32948,7 +33034,7 @@
         <v>1092</v>
       </c>
       <c r="L860" s="57" t="str">
-        <f t="shared" si="102"/>
+        <f t="shared" si="103"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0140_Goetterneunheit/epitheta/02_nDs.t/0040_nDs.t_Sp_01.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -33136,7 +33222,7 @@
         <v>765</v>
       </c>
       <c r="L874" s="57" t="str">
-        <f t="shared" ref="L874:L875" si="103">_xlfn.TEXTJOIN("", TRUE, D874:J874)</f>
+        <f t="shared" ref="L874:L875" si="104">_xlfn.TEXTJOIN("", TRUE, D874:J874)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0160_Maat/0001_mAa.t_01.png</v>
       </c>
     </row>
@@ -33157,7 +33243,7 @@
         <v>766</v>
       </c>
       <c r="L875" s="57" t="str">
-        <f t="shared" si="103"/>
+        <f t="shared" si="104"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0160_Maat/0010_mAa.t_02.png</v>
       </c>
     </row>
@@ -33187,7 +33273,7 @@
         <v>1092</v>
       </c>
       <c r="L876" s="57" t="str">
-        <f t="shared" ref="L876:L885" si="104">_xlfn.TEXTJOIN("", TRUE, D876:K876)</f>
+        <f t="shared" ref="L876:L885" si="105">_xlfn.TEXTJOIN("", TRUE, D876:K876)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0160_Maat/0020_mAa.t_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -33217,7 +33303,7 @@
         <v>1092</v>
       </c>
       <c r="L877" s="57" t="str">
-        <f t="shared" si="104"/>
+        <f t="shared" si="105"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0160_Maat/0030_mAa.t_AR_02.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -33247,7 +33333,7 @@
         <v>1092</v>
       </c>
       <c r="L878" s="57" t="str">
-        <f t="shared" si="104"/>
+        <f t="shared" si="105"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0160_Maat/0040_mAa.t_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -33277,7 +33363,7 @@
         <v>1092</v>
       </c>
       <c r="L879" s="57" t="str">
-        <f t="shared" si="104"/>
+        <f t="shared" si="105"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0160_Maat/0050_mAa.t_MR_02.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -33307,7 +33393,7 @@
         <v>1092</v>
       </c>
       <c r="L880" s="57" t="str">
-        <f t="shared" si="104"/>
+        <f t="shared" si="105"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0160_Maat/0060_mAa.t_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -33337,7 +33423,7 @@
         <v>1092</v>
       </c>
       <c r="L881" s="57" t="str">
-        <f t="shared" si="104"/>
+        <f t="shared" si="105"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0160_Maat/0070_mAa.t_NR_02.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -33367,7 +33453,7 @@
         <v>1092</v>
       </c>
       <c r="L882" s="57" t="str">
-        <f t="shared" si="104"/>
+        <f t="shared" si="105"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0160_Maat/0080_mAa.t_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -33397,7 +33483,7 @@
         <v>1092</v>
       </c>
       <c r="L883" s="57" t="str">
-        <f t="shared" si="104"/>
+        <f t="shared" si="105"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0160_Maat/0090_mAa.t_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -33430,7 +33516,7 @@
         <v>1092</v>
       </c>
       <c r="L884" s="57" t="str">
-        <f t="shared" si="104"/>
+        <f t="shared" si="105"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0160_Maat/det/0001_mAa.t_det_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -33463,7 +33549,7 @@
         <v>1092</v>
       </c>
       <c r="L885" s="57" t="str">
-        <f t="shared" si="104"/>
+        <f t="shared" si="105"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0160_Maat/det/0010_mAa.t_det_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -33928,7 +34014,7 @@
         <v>790</v>
       </c>
       <c r="L921" s="57" t="str">
-        <f t="shared" ref="L921:L927" si="105">_xlfn.TEXTJOIN("", TRUE, D921:J921)</f>
+        <f t="shared" ref="L921:L927" si="106">_xlfn.TEXTJOIN("", TRUE, D921:J921)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0190_Month/0001_mnTw_01.png</v>
       </c>
     </row>
@@ -33988,7 +34074,7 @@
         <v>1092</v>
       </c>
       <c r="L923" s="57" t="str">
-        <f t="shared" ref="L923:L925" si="106">_xlfn.TEXTJOIN("", TRUE, D923:K923)</f>
+        <f t="shared" ref="L923:L925" si="107">_xlfn.TEXTJOIN("", TRUE, D923:K923)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0190_Month/0020_mnTw_NR_02.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -34018,7 +34104,7 @@
         <v>1092</v>
       </c>
       <c r="L924" s="57" t="str">
-        <f t="shared" si="106"/>
+        <f t="shared" si="107"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0190_Month/0030_mnTw_NR_03.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -34048,7 +34134,7 @@
         <v>1092</v>
       </c>
       <c r="L925" s="57" t="str">
-        <f t="shared" si="106"/>
+        <f t="shared" si="107"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0190_Month/0040_mnTw_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -34072,7 +34158,7 @@
         <v>795</v>
       </c>
       <c r="L926" s="57" t="str">
-        <f t="shared" si="105"/>
+        <f t="shared" si="106"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0190_Month/det/0001_mnTw_det_01.png</v>
       </c>
     </row>
@@ -34096,7 +34182,7 @@
         <v>796</v>
       </c>
       <c r="L927" s="57" t="str">
-        <f t="shared" si="105"/>
+        <f t="shared" si="106"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0190_Month/det/0010_mnTw_det_02.png</v>
       </c>
     </row>
@@ -34176,7 +34262,7 @@
         <v>801</v>
       </c>
       <c r="L933" s="57" t="str">
-        <f t="shared" ref="L933:L940" si="107">_xlfn.TEXTJOIN("", TRUE, D933:K933)</f>
+        <f t="shared" ref="L933:L940" si="108">_xlfn.TEXTJOIN("", TRUE, D933:K933)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0190_Month/epitheta/01_nb-wAs.t/0001_nb-WAs.t_01.png</v>
       </c>
     </row>
@@ -34209,7 +34295,7 @@
         <v>1092</v>
       </c>
       <c r="L934" s="57" t="str">
-        <f t="shared" si="107"/>
+        <f t="shared" si="108"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0190_Month/epitheta/01_nb-wAs.t/0010_nb-WAs.t_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -34242,7 +34328,7 @@
         <v>1092</v>
       </c>
       <c r="L935" s="57" t="str">
-        <f t="shared" si="107"/>
+        <f t="shared" si="108"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0190_Month/epitheta/01_nb-wAs.t/0020_nb-WAs.t_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -34275,7 +34361,7 @@
         <v>1092</v>
       </c>
       <c r="L936" s="57" t="str">
-        <f t="shared" si="107"/>
+        <f t="shared" si="108"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0190_Month/epitheta/01_nb-wAs.t/0030_nb-WAs.t_NR_02.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -34308,7 +34394,7 @@
         <v>1092</v>
       </c>
       <c r="L937" s="57" t="str">
-        <f t="shared" si="107"/>
+        <f t="shared" si="108"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0190_Month/epitheta/01_nb-wAs.t/0040_nb-WAs.t_NR_03.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -34344,7 +34430,7 @@
         <v>1092</v>
       </c>
       <c r="L938" s="57" t="str">
-        <f t="shared" si="107"/>
+        <f t="shared" si="108"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0190_Month/epitheta/01_nb-wAs.t/0050_nb-WAs.t_NR_04.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -34380,7 +34466,7 @@
         <v>1092</v>
       </c>
       <c r="L939" s="57" t="str">
-        <f t="shared" si="107"/>
+        <f t="shared" si="108"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0190_Month/epitheta/01_nb-wAs.t/0060_nb-WAs.t_Sp_01.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -34416,7 +34502,7 @@
         <v>1092</v>
       </c>
       <c r="L940" s="57" t="str">
-        <f t="shared" si="107"/>
+        <f t="shared" si="108"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0190_Month/epitheta/01_nb-wAs.t/0070_nb-WAs.t_Gr_01.png &lt;sup&gt;  &lt;/sup&gt;</v>
       </c>
     </row>
@@ -34587,7 +34673,7 @@
         <v>105</v>
       </c>
       <c r="L952" s="57" t="str">
-        <f t="shared" ref="L952" si="108">_xlfn.TEXTJOIN("", TRUE, D952:J952)</f>
+        <f t="shared" ref="L952" si="109">_xlfn.TEXTJOIN("", TRUE, D952:J952)</f>
         <v/>
       </c>
     </row>
@@ -34661,7 +34747,7 @@
         <v>811</v>
       </c>
       <c r="L959" s="57" t="str">
-        <f t="shared" ref="L959:L964" si="109">_xlfn.TEXTJOIN("", TRUE, D959:K959)</f>
+        <f t="shared" ref="L959:L964" si="110">_xlfn.TEXTJOIN("", TRUE, D959:K959)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0210_Nut/0001_nw.t_01.png</v>
       </c>
     </row>
@@ -34691,7 +34777,7 @@
         <v>1092</v>
       </c>
       <c r="L960" s="57" t="str">
-        <f t="shared" si="109"/>
+        <f t="shared" si="110"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0210_Nut/0010_nw.t_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -34721,7 +34807,7 @@
         <v>1092</v>
       </c>
       <c r="L961" s="57" t="str">
-        <f t="shared" si="109"/>
+        <f t="shared" si="110"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0210_Nut/0020_nw.t_AR_02.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -34751,7 +34837,7 @@
         <v>1092</v>
       </c>
       <c r="L962" s="57" t="str">
-        <f t="shared" si="109"/>
+        <f t="shared" si="110"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0210_Nut/0030_nw.t_AR_03.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -34781,7 +34867,7 @@
         <v>1092</v>
       </c>
       <c r="L963" s="57" t="str">
-        <f t="shared" si="109"/>
+        <f t="shared" si="110"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0210_Nut/0040_nw.t_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -34811,7 +34897,7 @@
         <v>1092</v>
       </c>
       <c r="L964" s="57" t="str">
-        <f t="shared" si="109"/>
+        <f t="shared" si="110"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0210_Nut/0050_nw.t_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -34826,7 +34912,7 @@
         <v>105</v>
       </c>
       <c r="L965" s="57" t="str">
-        <f t="shared" ref="L965" si="110">_xlfn.TEXTJOIN("", TRUE, D965:J965)</f>
+        <f t="shared" ref="L965" si="111">_xlfn.TEXTJOIN("", TRUE, D965:J965)</f>
         <v/>
       </c>
     </row>
@@ -34900,7 +34986,7 @@
         <v>817</v>
       </c>
       <c r="L972" s="57" t="str">
-        <f t="shared" ref="L972:L978" si="111">_xlfn.TEXTJOIN("", TRUE, D972:K972)</f>
+        <f t="shared" ref="L972:L978" si="112">_xlfn.TEXTJOIN("", TRUE, D972:K972)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0220_Nephthys/0001_nb.t-Hw.t_01.png</v>
       </c>
     </row>
@@ -34930,7 +35016,7 @@
         <v>1092</v>
       </c>
       <c r="L973" s="57" t="str">
-        <f t="shared" si="111"/>
+        <f t="shared" si="112"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0220_Nephthys/0010_nb.t-Hw.t_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -34960,7 +35046,7 @@
         <v>1092</v>
       </c>
       <c r="L974" s="57" t="str">
-        <f t="shared" si="111"/>
+        <f t="shared" si="112"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0220_Nephthys/0020_nb.t-Hw.t_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -34990,7 +35076,7 @@
         <v>1092</v>
       </c>
       <c r="L975" s="57" t="str">
-        <f t="shared" si="111"/>
+        <f t="shared" si="112"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0220_Nephthys/0030_nb.t-Hw.t_NR_02.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -35020,7 +35106,7 @@
         <v>1092</v>
       </c>
       <c r="L976" s="57" t="str">
-        <f t="shared" si="111"/>
+        <f t="shared" si="112"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0220_Nephthys/0040_nb.t-Hw.t_SP_01.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -35050,7 +35136,7 @@
         <v>1092</v>
       </c>
       <c r="L977" s="57" t="str">
-        <f t="shared" si="111"/>
+        <f t="shared" si="112"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0220_Nephthys/0050_nb.t-Hw.t_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -35080,7 +35166,7 @@
         <v>1092</v>
       </c>
       <c r="L978" s="57" t="str">
-        <f t="shared" si="111"/>
+        <f t="shared" si="112"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0220_Nephthys/0060_nb.t-Hw.t_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -35095,7 +35181,7 @@
         <v>105</v>
       </c>
       <c r="L979" s="57" t="str">
-        <f t="shared" ref="L979" si="112">_xlfn.TEXTJOIN("", TRUE, D979:J979)</f>
+        <f t="shared" ref="L979" si="113">_xlfn.TEXTJOIN("", TRUE, D979:J979)</f>
         <v/>
       </c>
     </row>
@@ -35169,7 +35255,7 @@
         <v>824</v>
       </c>
       <c r="L986" s="57" t="str">
-        <f t="shared" ref="L986:L987" si="113">_xlfn.TEXTJOIN("", TRUE, D986:J986)</f>
+        <f t="shared" ref="L986:L987" si="114">_xlfn.TEXTJOIN("", TRUE, D986:J986)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0230_Nefertem/0001_nfr-tm_01.png</v>
       </c>
     </row>
@@ -35190,7 +35276,7 @@
         <v>825</v>
       </c>
       <c r="L987" s="57" t="str">
-        <f t="shared" si="113"/>
+        <f t="shared" si="114"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0230_Nefertem/0010_nfr-tm_02.png</v>
       </c>
     </row>
@@ -35220,7 +35306,7 @@
         <v>1092</v>
       </c>
       <c r="L988" s="57" t="str">
-        <f t="shared" ref="L988:L992" si="114">_xlfn.TEXTJOIN("", TRUE, D988:K988)</f>
+        <f t="shared" ref="L988:L992" si="115">_xlfn.TEXTJOIN("", TRUE, D988:K988)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0230_Nefertem/0020_nfr-tm_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -35250,7 +35336,7 @@
         <v>1092</v>
       </c>
       <c r="L989" s="57" t="str">
-        <f t="shared" si="114"/>
+        <f t="shared" si="115"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0230_Nefertem/0030_nfr-tm_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -35280,7 +35366,7 @@
         <v>1092</v>
       </c>
       <c r="L990" s="57" t="str">
-        <f t="shared" si="114"/>
+        <f t="shared" si="115"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0230_Nefertem/0040_nfr-tm_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -35313,7 +35399,7 @@
         <v>1092</v>
       </c>
       <c r="L991" s="57" t="str">
-        <f t="shared" si="114"/>
+        <f t="shared" si="115"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0230_Nefertem/det/0001_nfr-tm_det_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -35346,7 +35432,7 @@
         <v>1092</v>
       </c>
       <c r="L992" s="57" t="str">
-        <f t="shared" si="114"/>
+        <f t="shared" si="115"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0230_Nefertem/det/0010_nfr-tm_det_NR_02.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -35471,7 +35557,7 @@
         <v>1092</v>
       </c>
       <c r="L1001" s="57" t="str">
-        <f t="shared" ref="L1001:L1003" si="115">_xlfn.TEXTJOIN("", TRUE, D1001:K1001)</f>
+        <f t="shared" ref="L1001:L1003" si="116">_xlfn.TEXTJOIN("", TRUE, D1001:K1001)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0240_Nechbet/0020_nxb.t_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -35501,7 +35587,7 @@
         <v>1092</v>
       </c>
       <c r="L1002" s="57" t="str">
-        <f t="shared" si="115"/>
+        <f t="shared" si="116"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0240_Nechbet/0030_nxb.t_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -35537,7 +35623,7 @@
         <v>1092</v>
       </c>
       <c r="L1003" s="57" t="str">
-        <f t="shared" si="115"/>
+        <f t="shared" si="116"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0240_Nechbet/det/0001_nxb.t_det_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -35611,7 +35697,7 @@
         <v>836</v>
       </c>
       <c r="L1010" s="57" t="str">
-        <f t="shared" ref="L1010" si="116">_xlfn.TEXTJOIN("", TRUE, D1010:J1010)</f>
+        <f t="shared" ref="L1010" si="117">_xlfn.TEXTJOIN("", TRUE, D1010:J1010)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0250_Re/0001_ra_01.png</v>
       </c>
     </row>
@@ -35641,7 +35727,7 @@
         <v>1092</v>
       </c>
       <c r="L1011" s="57" t="str">
-        <f t="shared" ref="L1011:L1017" si="117">_xlfn.TEXTJOIN("", TRUE, D1011:K1011)</f>
+        <f t="shared" ref="L1011:L1017" si="118">_xlfn.TEXTJOIN("", TRUE, D1011:K1011)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0250_Re/0010_ra_SP_01.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -35671,7 +35757,7 @@
         <v>1092</v>
       </c>
       <c r="L1012" s="57" t="str">
-        <f t="shared" si="117"/>
+        <f t="shared" si="118"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0250_Re/0020_ra_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -35701,7 +35787,7 @@
         <v>1092</v>
       </c>
       <c r="L1013" s="57" t="str">
-        <f t="shared" si="117"/>
+        <f t="shared" si="118"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0250_Re/0030_ra_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -35734,7 +35820,7 @@
         <v>1092</v>
       </c>
       <c r="L1014" s="57" t="str">
-        <f t="shared" si="117"/>
+        <f t="shared" si="118"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0250_Re/det/0001_ra_det_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -35767,7 +35853,7 @@
         <v>1092</v>
       </c>
       <c r="L1015" s="57" t="str">
-        <f t="shared" si="117"/>
+        <f t="shared" si="118"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0250_Re/det/0010_ra_det_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -35800,7 +35886,7 @@
         <v>1092</v>
       </c>
       <c r="L1016" s="57" t="str">
-        <f t="shared" si="117"/>
+        <f t="shared" si="118"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0250_Re/det/0020_ra_det_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -35833,7 +35919,7 @@
         <v>1092</v>
       </c>
       <c r="L1017" s="57" t="str">
-        <f t="shared" si="117"/>
+        <f t="shared" si="118"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0250_Re/det/0030_ra_det_NR_02.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -35993,7 +36079,7 @@
         <v>844</v>
       </c>
       <c r="L1032" s="57" t="str">
-        <f t="shared" ref="L1032:L1038" si="118">_xlfn.TEXTJOIN("", TRUE, D1032:J1032)</f>
+        <f t="shared" ref="L1032:L1038" si="119">_xlfn.TEXTJOIN("", TRUE, D1032:J1032)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0270_Renenutet/0001_rnnwt.t_01.png</v>
       </c>
     </row>
@@ -36023,7 +36109,7 @@
         <v>1092</v>
       </c>
       <c r="L1033" s="57" t="str">
-        <f t="shared" ref="L1033:L1037" si="119">_xlfn.TEXTJOIN("", TRUE, D1033:K1033)</f>
+        <f t="shared" ref="L1033:L1037" si="120">_xlfn.TEXTJOIN("", TRUE, D1033:K1033)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0270_Renenutet/0010_rnnwt.t_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -36053,7 +36139,7 @@
         <v>1092</v>
       </c>
       <c r="L1034" s="57" t="str">
-        <f t="shared" si="119"/>
+        <f t="shared" si="120"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0270_Renenutet/0020_rnnwt.t_AR_02.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -36083,7 +36169,7 @@
         <v>1092</v>
       </c>
       <c r="L1035" s="57" t="str">
-        <f t="shared" si="119"/>
+        <f t="shared" si="120"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0270_Renenutet/0030_rnnwt.t_D.18_01.png &lt;sup&gt;(D.18)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -36113,7 +36199,7 @@
         <v>1092</v>
       </c>
       <c r="L1036" s="57" t="str">
-        <f t="shared" si="119"/>
+        <f t="shared" si="120"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0270_Renenutet/0040_rnnwt.t_D.18_02.png &lt;sup&gt;(D.18)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -36143,7 +36229,7 @@
         <v>1092</v>
       </c>
       <c r="L1037" s="57" t="str">
-        <f t="shared" si="119"/>
+        <f t="shared" si="120"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0270_Renenutet/0050_rnnwt.t_D.18_03.png &lt;sup&gt;(D.18)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -36158,7 +36244,7 @@
         <v>105</v>
       </c>
       <c r="L1038" s="57" t="str">
-        <f t="shared" si="118"/>
+        <f t="shared" si="119"/>
         <v/>
       </c>
     </row>
@@ -36241,7 +36327,7 @@
         <v>1092</v>
       </c>
       <c r="L1045" s="57" t="str">
-        <f t="shared" ref="L1045:L1056" si="120">_xlfn.TEXTJOIN("", TRUE, D1045:K1045)</f>
+        <f t="shared" ref="L1045:L1056" si="121">_xlfn.TEXTJOIN("", TRUE, D1045:K1045)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0280_Hapi-Nilgott/0001_Hapj_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -36271,7 +36357,7 @@
         <v>1092</v>
       </c>
       <c r="L1046" s="57" t="str">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0280_Hapi-Nilgott/0010_Hapj_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -36301,7 +36387,7 @@
         <v>1092</v>
       </c>
       <c r="L1047" s="57" t="str">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0280_Hapi-Nilgott/0020_Hapj_MR_02.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -36331,7 +36417,7 @@
         <v>1092</v>
       </c>
       <c r="L1048" s="57" t="str">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0280_Hapi-Nilgott/0030_Hapj_MR_03.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -36361,7 +36447,7 @@
         <v>1092</v>
       </c>
       <c r="L1049" s="57" t="str">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0280_Hapi-Nilgott/0040_Hapj_MR_04.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -36391,7 +36477,7 @@
         <v>1092</v>
       </c>
       <c r="L1050" s="57" t="str">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0280_Hapi-Nilgott/0050_Hapj_MR_05.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -36421,7 +36507,7 @@
         <v>1092</v>
       </c>
       <c r="L1051" s="57" t="str">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0280_Hapi-Nilgott/0060_Hapj_MR_06.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -36451,7 +36537,7 @@
         <v>1092</v>
       </c>
       <c r="L1052" s="57" t="str">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0280_Hapi-Nilgott/0070_Hapj_Sait._01.png &lt;sup&gt;(Saït.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -36481,7 +36567,7 @@
         <v>1092</v>
       </c>
       <c r="L1053" s="57" t="str">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0280_Hapi-Nilgott/0080_Hapj_Sait._02.png &lt;sup&gt;(Saït.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -36511,7 +36597,7 @@
         <v>1092</v>
       </c>
       <c r="L1054" s="57" t="str">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0280_Hapi-Nilgott/0090_Hapj_SP-GR_01.png &lt;sup&gt;(Sp.–Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -36541,7 +36627,7 @@
         <v>1092</v>
       </c>
       <c r="L1055" s="57" t="str">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0280_Hapi-Nilgott/0100_Hapj_SP-GR_02.png &lt;sup&gt;(Sp.–Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -36571,7 +36657,7 @@
         <v>1092</v>
       </c>
       <c r="L1056" s="57" t="str">
-        <f t="shared" si="120"/>
+        <f t="shared" si="121"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0280_Hapi-Nilgott/0110_Hapj_SP-GR_03.png &lt;sup&gt;(Sp.–Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -36595,7 +36681,7 @@
         <v>859</v>
       </c>
       <c r="L1057" s="57" t="str">
-        <f t="shared" ref="L1057:L1058" si="121">_xlfn.TEXTJOIN("", TRUE, D1057:J1057)</f>
+        <f t="shared" ref="L1057:L1058" si="122">_xlfn.TEXTJOIN("", TRUE, D1057:J1057)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0280_Hapi-Nilgott/det/0001_Hapj_det_01.png</v>
       </c>
     </row>
@@ -36619,7 +36705,7 @@
         <v>860</v>
       </c>
       <c r="L1058" s="57" t="str">
-        <f t="shared" si="121"/>
+        <f t="shared" si="122"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0280_Hapi-Nilgott/det/0010_Hapj_det_02.png</v>
       </c>
     </row>
@@ -36723,7 +36809,7 @@
         <v>1092</v>
       </c>
       <c r="L1066" s="57" t="str">
-        <f t="shared" ref="L1066:L1067" si="122">_xlfn.TEXTJOIN("", TRUE, D1066:K1066)</f>
+        <f t="shared" ref="L1066:L1067" si="123">_xlfn.TEXTJOIN("", TRUE, D1066:K1066)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0290_Hathor/0010_Hwt-Hr_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -36753,7 +36839,7 @@
         <v>1092</v>
       </c>
       <c r="L1067" s="57" t="str">
-        <f t="shared" si="122"/>
+        <f t="shared" si="123"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0290_Hathor/0020_Hwt-Hr_AR_02.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -36842,7 +36928,7 @@
         <v>867</v>
       </c>
       <c r="L1075" s="57" t="str">
-        <f t="shared" ref="L1075:L1080" si="123">_xlfn.TEXTJOIN("", TRUE, D1075:J1075)</f>
+        <f t="shared" ref="L1075:L1080" si="124">_xlfn.TEXTJOIN("", TRUE, D1075:J1075)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0300_Apis/0001_Hp_01.png</v>
       </c>
     </row>
@@ -36863,7 +36949,7 @@
         <v>868</v>
       </c>
       <c r="L1076" s="57" t="str">
-        <f t="shared" si="123"/>
+        <f t="shared" si="124"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0300_Apis/0010_Hp_02.png</v>
       </c>
     </row>
@@ -36893,7 +36979,7 @@
         <v>1092</v>
       </c>
       <c r="L1077" s="57" t="str">
-        <f t="shared" ref="L1077:L1078" si="124">_xlfn.TEXTJOIN("", TRUE, D1077:K1077)</f>
+        <f t="shared" ref="L1077:L1078" si="125">_xlfn.TEXTJOIN("", TRUE, D1077:K1077)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0300_Apis/0020_Hp_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -36923,7 +37009,7 @@
         <v>1092</v>
       </c>
       <c r="L1078" s="57" t="str">
-        <f t="shared" si="124"/>
+        <f t="shared" si="125"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0300_Apis/0030_Hp_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -36947,7 +37033,7 @@
         <v>871</v>
       </c>
       <c r="L1079" s="57" t="str">
-        <f t="shared" si="123"/>
+        <f t="shared" si="124"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0300_Apis/det/0001_Hp_det_01.png</v>
       </c>
     </row>
@@ -36971,7 +37057,7 @@
         <v>872</v>
       </c>
       <c r="L1080" s="57" t="str">
-        <f t="shared" si="123"/>
+        <f t="shared" si="124"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0300_Apis/det/0010_Hp_det_02.png</v>
       </c>
     </row>
@@ -37159,7 +37245,7 @@
         <v>877</v>
       </c>
       <c r="L1096" s="57" t="str">
-        <f t="shared" ref="L1096:L1104" si="125">_xlfn.TEXTJOIN("", TRUE, D1096:J1096)</f>
+        <f t="shared" ref="L1096:L1104" si="126">_xlfn.TEXTJOIN("", TRUE, D1096:J1096)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0310_Hapi-Horussohn/0001_Hpy_01.png</v>
       </c>
     </row>
@@ -37180,7 +37266,7 @@
         <v>878</v>
       </c>
       <c r="L1097" s="57" t="str">
-        <f t="shared" si="125"/>
+        <f t="shared" si="126"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0310_Hapi-Horussohn/0010_Hpy_02.png</v>
       </c>
     </row>
@@ -37201,7 +37287,7 @@
         <v>879</v>
       </c>
       <c r="L1098" s="57" t="str">
-        <f t="shared" si="125"/>
+        <f t="shared" si="126"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0310_Hapi-Horussohn/0020_Hpy_03.png</v>
       </c>
     </row>
@@ -37222,7 +37308,7 @@
         <v>880</v>
       </c>
       <c r="L1099" s="57" t="str">
-        <f t="shared" si="125"/>
+        <f t="shared" si="126"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0310_Hapi-Horussohn/0030_Hpy_04.png</v>
       </c>
     </row>
@@ -37252,7 +37338,7 @@
         <v>1092</v>
       </c>
       <c r="L1100" s="57" t="str">
-        <f t="shared" ref="L1100:L1102" si="126">_xlfn.TEXTJOIN("", TRUE, D1100:K1100)</f>
+        <f t="shared" ref="L1100:L1102" si="127">_xlfn.TEXTJOIN("", TRUE, D1100:K1100)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0310_Hapi-Horussohn/0040_Hpy_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -37282,7 +37368,7 @@
         <v>1092</v>
       </c>
       <c r="L1101" s="57" t="str">
-        <f t="shared" si="126"/>
+        <f t="shared" si="127"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0310_Hapi-Horussohn/0050_Hpy_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -37312,7 +37398,7 @@
         <v>1092</v>
       </c>
       <c r="L1102" s="57" t="str">
-        <f t="shared" si="126"/>
+        <f t="shared" si="127"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0310_Hapi-Horussohn/0060_Hpy_MR-NR-GR_01.png &lt;sup&gt;(MR; NR; Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -37336,7 +37422,7 @@
         <v>884</v>
       </c>
       <c r="L1103" s="57" t="str">
-        <f t="shared" si="125"/>
+        <f t="shared" si="126"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0310_Hapi-Horussohn/det/0001_Hpy_det_01.png</v>
       </c>
     </row>
@@ -37360,7 +37446,7 @@
         <v>885</v>
       </c>
       <c r="L1104" s="57" t="str">
-        <f t="shared" si="125"/>
+        <f t="shared" si="126"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0310_Hapi-Horussohn/det/0010_Hpy_det_AR_01.png</v>
       </c>
     </row>
@@ -37485,7 +37571,7 @@
         <v>1092</v>
       </c>
       <c r="L1113" s="57" t="str">
-        <f t="shared" ref="L1113:L1114" si="127">_xlfn.TEXTJOIN("", TRUE, D1113:K1113)</f>
+        <f t="shared" ref="L1113:L1114" si="128">_xlfn.TEXTJOIN("", TRUE, D1113:K1113)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0320_Horus/0020_Hr_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -37515,7 +37601,7 @@
         <v>1092</v>
       </c>
       <c r="L1114" s="57" t="str">
-        <f t="shared" si="127"/>
+        <f t="shared" si="128"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0320_Horus/0030_Hr_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -38313,7 +38399,7 @@
         <v>914</v>
       </c>
       <c r="L1171" s="57" t="str">
-        <f t="shared" ref="L1171:L1178" si="128">_xlfn.TEXTJOIN("", TRUE, D1171:J1171)</f>
+        <f t="shared" ref="L1171:L1178" si="129">_xlfn.TEXTJOIN("", TRUE, D1171:J1171)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0350_Chnum/0001_Xnm.w_01.png</v>
       </c>
     </row>
@@ -38334,7 +38420,7 @@
         <v>915</v>
       </c>
       <c r="L1172" s="57" t="str">
-        <f t="shared" si="128"/>
+        <f t="shared" si="129"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0350_Chnum/0010_Xnm.w_02.png</v>
       </c>
     </row>
@@ -38355,7 +38441,7 @@
         <v>916</v>
       </c>
       <c r="L1173" s="57" t="str">
-        <f t="shared" si="128"/>
+        <f t="shared" si="129"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0350_Chnum/0020_Xnm.w_03.png</v>
       </c>
     </row>
@@ -38376,7 +38462,7 @@
         <v>917</v>
       </c>
       <c r="L1174" s="57" t="str">
-        <f t="shared" si="128"/>
+        <f t="shared" si="129"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0350_Chnum/0030_Xnm.w_04.png</v>
       </c>
     </row>
@@ -38406,7 +38492,7 @@
         <v>1092</v>
       </c>
       <c r="L1175" s="57" t="str">
-        <f t="shared" ref="L1175:L1176" si="129">_xlfn.TEXTJOIN("", TRUE, D1175:K1175)</f>
+        <f t="shared" ref="L1175:L1176" si="130">_xlfn.TEXTJOIN("", TRUE, D1175:K1175)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0350_Chnum/0040_Xnm.w_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -38436,7 +38522,7 @@
         <v>1092</v>
       </c>
       <c r="L1176" s="57" t="str">
-        <f t="shared" si="129"/>
+        <f t="shared" si="130"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0350_Chnum/0050_Xnm.w_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -38460,7 +38546,7 @@
         <v>920</v>
       </c>
       <c r="L1177" s="57" t="str">
-        <f t="shared" si="128"/>
+        <f t="shared" si="129"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0350_Chnum/det/0001_Xnm.w_det_01.png</v>
       </c>
     </row>
@@ -38484,7 +38570,7 @@
         <v>921</v>
       </c>
       <c r="L1178" s="57" t="str">
-        <f t="shared" si="128"/>
+        <f t="shared" si="129"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0350_Chnum/det/0010_Xnm.w_det_02.png</v>
       </c>
     </row>
@@ -38558,7 +38644,7 @@
         <v>922</v>
       </c>
       <c r="L1185" s="57" t="str">
-        <f t="shared" ref="L1185:L1186" si="130">_xlfn.TEXTJOIN("", TRUE, D1185:K1185)</f>
+        <f t="shared" ref="L1185:L1186" si="131">_xlfn.TEXTJOIN("", TRUE, D1185:K1185)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0360_Chons/0001_Xnsw_01.png</v>
       </c>
     </row>
@@ -38579,7 +38665,7 @@
         <v>923</v>
       </c>
       <c r="L1186" s="57" t="str">
-        <f t="shared" si="130"/>
+        <f t="shared" si="131"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0360_Chons/0010_Xnsw_02.png</v>
       </c>
     </row>
@@ -38716,7 +38802,7 @@
         <v>1092</v>
       </c>
       <c r="L1194" s="57" t="str">
-        <f t="shared" ref="L1194:L1195" si="131">_xlfn.TEXTJOIN("", TRUE, D1194:K1194)</f>
+        <f t="shared" ref="L1194:L1195" si="132">_xlfn.TEXTJOIN("", TRUE, D1194:K1194)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0360_Chons/epitheta/01-m-wAs.t/0001_m-WAs.t_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -38749,7 +38835,7 @@
         <v>1092</v>
       </c>
       <c r="L1195" s="57" t="str">
-        <f t="shared" si="131"/>
+        <f t="shared" si="132"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0360_Chons/epitheta/01-m-wAs.t/0010_m-WAs.t_NR_02.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -38827,7 +38913,7 @@
         <v>1092</v>
       </c>
       <c r="L1200" s="57" t="str">
-        <f t="shared" ref="L1200" si="132">_xlfn.TEXTJOIN("", TRUE, D1200:K1200)</f>
+        <f t="shared" ref="L1200" si="133">_xlfn.TEXTJOIN("", TRUE, D1200:K1200)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0360_Chons/epitheta/02-pA-jrj-sxr.w-m-WAs.t/0001_pA-jrj-sxr.w-m-WAs.t_Sp_01.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -39072,7 +39158,7 @@
         <v>930</v>
       </c>
       <c r="L1221" s="57" t="str">
-        <f t="shared" ref="L1221:L1229" si="133">_xlfn.TEXTJOIN("", TRUE, D1221:J1221)</f>
+        <f t="shared" ref="L1221:L1229" si="134">_xlfn.TEXTJOIN("", TRUE, D1221:J1221)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/0001_srq.t_01.png</v>
       </c>
     </row>
@@ -39093,7 +39179,7 @@
         <v>931</v>
       </c>
       <c r="L1222" s="57" t="str">
-        <f t="shared" si="133"/>
+        <f t="shared" si="134"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/0010_srq.t_02.png</v>
       </c>
     </row>
@@ -39114,7 +39200,7 @@
         <v>932</v>
       </c>
       <c r="L1223" s="57" t="str">
-        <f t="shared" si="133"/>
+        <f t="shared" si="134"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/0020_srq.t_03.png</v>
       </c>
     </row>
@@ -39144,7 +39230,7 @@
         <v>1092</v>
       </c>
       <c r="L1224" s="57" t="str">
-        <f t="shared" ref="L1224:L1227" si="134">_xlfn.TEXTJOIN("", TRUE, D1224:K1224)</f>
+        <f t="shared" ref="L1224:L1227" si="135">_xlfn.TEXTJOIN("", TRUE, D1224:K1224)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/0030_srq.t_Pyr.-MR_01.png &lt;sup&gt;(Pyr.; NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -39174,7 +39260,7 @@
         <v>1092</v>
       </c>
       <c r="L1225" s="57" t="str">
-        <f t="shared" si="134"/>
+        <f t="shared" si="135"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/0040_srq.t_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -39204,7 +39290,7 @@
         <v>1092</v>
       </c>
       <c r="L1226" s="57" t="str">
-        <f t="shared" si="134"/>
+        <f t="shared" si="135"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/0050_srq.t_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -39234,7 +39320,7 @@
         <v>1092</v>
       </c>
       <c r="L1227" s="57" t="str">
-        <f t="shared" si="134"/>
+        <f t="shared" si="135"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/0060_srq.t_GR_03.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -39258,7 +39344,7 @@
         <v>937</v>
       </c>
       <c r="L1228" s="57" t="str">
-        <f t="shared" si="133"/>
+        <f t="shared" si="134"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/det/0001_srq.t_det_01.png</v>
       </c>
     </row>
@@ -39282,7 +39368,7 @@
         <v>938</v>
       </c>
       <c r="L1229" s="57" t="str">
-        <f t="shared" si="133"/>
+        <f t="shared" si="134"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/det/0010_srq.t_det_02.png</v>
       </c>
     </row>
@@ -39356,7 +39442,7 @@
         <v>939</v>
       </c>
       <c r="L1236" s="57" t="str">
-        <f t="shared" ref="L1236:L1242" si="135">_xlfn.TEXTJOIN("", TRUE, D1236:J1236)</f>
+        <f t="shared" ref="L1236:L1242" si="136">_xlfn.TEXTJOIN("", TRUE, D1236:J1236)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0390_Sachmet/0001_sxm.t_01.png</v>
       </c>
     </row>
@@ -39386,7 +39472,7 @@
         <v>1092</v>
       </c>
       <c r="L1237" s="57" t="str">
-        <f t="shared" ref="L1237:L1241" si="136">_xlfn.TEXTJOIN("", TRUE, D1237:K1237)</f>
+        <f t="shared" ref="L1237:L1241" si="137">_xlfn.TEXTJOIN("", TRUE, D1237:K1237)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0390_Sachmet/0010_sxm.t_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -39416,7 +39502,7 @@
         <v>1092</v>
       </c>
       <c r="L1238" s="57" t="str">
-        <f t="shared" si="136"/>
+        <f t="shared" si="137"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0390_Sachmet/0020_sxm.t_AR_02.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -39446,7 +39532,7 @@
         <v>1092</v>
       </c>
       <c r="L1239" s="57" t="str">
-        <f t="shared" si="136"/>
+        <f t="shared" si="137"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0390_Sachmet/0030_sxm.t_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -39476,7 +39562,7 @@
         <v>1092</v>
       </c>
       <c r="L1240" s="57" t="str">
-        <f t="shared" si="136"/>
+        <f t="shared" si="137"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0390_Sachmet/0040_sxm.t_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -39506,7 +39592,7 @@
         <v>1092</v>
       </c>
       <c r="L1241" s="57" t="str">
-        <f t="shared" si="136"/>
+        <f t="shared" si="137"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0390_Sachmet/0050_sxm.t_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -39521,7 +39607,7 @@
         <v>105</v>
       </c>
       <c r="L1242" s="57" t="str">
-        <f t="shared" si="135"/>
+        <f t="shared" si="136"/>
         <v/>
       </c>
     </row>
@@ -39693,7 +39779,7 @@
         <v>963</v>
       </c>
       <c r="L1257" s="57" t="str">
-        <f t="shared" ref="L1257:L1270" si="137">_xlfn.TEXTJOIN("", TRUE, D1257:J1257)</f>
+        <f t="shared" ref="L1257:L1270" si="138">_xlfn.TEXTJOIN("", TRUE, D1257:J1257)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0001_stX_01.png</v>
       </c>
     </row>
@@ -39723,7 +39809,7 @@
         <v>1092</v>
       </c>
       <c r="L1258" s="57" t="str">
-        <f t="shared" ref="L1258:L1268" si="138">_xlfn.TEXTJOIN("", TRUE, D1258:K1258)</f>
+        <f t="shared" ref="L1258:L1268" si="139">_xlfn.TEXTJOIN("", TRUE, D1258:K1258)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0010_stX_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -39753,7 +39839,7 @@
         <v>1092</v>
       </c>
       <c r="L1259" s="57" t="str">
-        <f t="shared" si="138"/>
+        <f t="shared" si="139"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0020_stX_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -39783,7 +39869,7 @@
         <v>1092</v>
       </c>
       <c r="L1260" s="57" t="str">
-        <f t="shared" si="138"/>
+        <f t="shared" si="139"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0030_stX_MR-SP_01.png &lt;sup&gt;(MR; Sp.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -39813,7 +39899,7 @@
         <v>1092</v>
       </c>
       <c r="L1261" s="57" t="str">
-        <f t="shared" si="138"/>
+        <f t="shared" si="139"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0040_stX_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -39843,7 +39929,7 @@
         <v>1092</v>
       </c>
       <c r="L1262" s="57" t="str">
-        <f t="shared" si="138"/>
+        <f t="shared" si="139"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0050_stX_D.18_01.png &lt;sup&gt;(D.18)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -39873,7 +39959,7 @@
         <v>1092</v>
       </c>
       <c r="L1263" s="57" t="str">
-        <f t="shared" si="138"/>
+        <f t="shared" si="139"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0060_stX_D.18_02.png &lt;sup&gt;(D.18)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -39903,7 +39989,7 @@
         <v>1092</v>
       </c>
       <c r="L1264" s="57" t="str">
-        <f t="shared" si="138"/>
+        <f t="shared" si="139"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0070_stX_D.18_03.png &lt;sup&gt;(D.18)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -39933,7 +40019,7 @@
         <v>1092</v>
       </c>
       <c r="L1265" s="57" t="str">
-        <f t="shared" si="138"/>
+        <f t="shared" si="139"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0080_stX_D.19_01.png &lt;sup&gt;(D.19)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -39963,7 +40049,7 @@
         <v>1092</v>
       </c>
       <c r="L1266" s="57" t="str">
-        <f t="shared" si="138"/>
+        <f t="shared" si="139"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0090_stX_D.19_02.png &lt;sup&gt;(D.19)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -39993,7 +40079,7 @@
         <v>1092</v>
       </c>
       <c r="L1267" s="57" t="str">
-        <f t="shared" si="138"/>
+        <f t="shared" si="139"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0100_stX_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -40023,7 +40109,7 @@
         <v>1092</v>
       </c>
       <c r="L1268" s="57" t="str">
-        <f t="shared" si="138"/>
+        <f t="shared" si="139"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0110_stX_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -40047,7 +40133,7 @@
         <v>974</v>
       </c>
       <c r="L1269" s="57" t="str">
-        <f t="shared" si="137"/>
+        <f t="shared" si="138"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/det/0001_stX_det_01.png</v>
       </c>
     </row>
@@ -40071,7 +40157,7 @@
         <v>975</v>
       </c>
       <c r="L1270" s="57" t="str">
-        <f t="shared" si="137"/>
+        <f t="shared" si="138"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/det/0010_stX_det_02.png</v>
       </c>
     </row>
@@ -40178,7 +40264,7 @@
         <v>977</v>
       </c>
       <c r="L1278" s="57" t="str">
-        <f t="shared" ref="L1278:L1283" si="139">_xlfn.TEXTJOIN("", TRUE, D1278:J1278)</f>
+        <f t="shared" ref="L1278:L1283" si="140">_xlfn.TEXTJOIN("", TRUE, D1278:J1278)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0420_Schu/0001_Sw_01.png</v>
       </c>
     </row>
@@ -40208,7 +40294,7 @@
         <v>1092</v>
       </c>
       <c r="L1279" s="57" t="str">
-        <f t="shared" ref="L1279:L1282" si="140">_xlfn.TEXTJOIN("", TRUE, D1279:K1279)</f>
+        <f t="shared" ref="L1279:L1282" si="141">_xlfn.TEXTJOIN("", TRUE, D1279:K1279)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0420_Schu/0010_Sw_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -40238,7 +40324,7 @@
         <v>1092</v>
       </c>
       <c r="L1280" s="57" t="str">
-        <f t="shared" si="140"/>
+        <f t="shared" si="141"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0420_Schu/0020_Sw_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -40268,7 +40354,7 @@
         <v>1092</v>
       </c>
       <c r="L1281" s="57" t="str">
-        <f t="shared" si="140"/>
+        <f t="shared" si="141"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0420_Schu/0030_Sw_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -40298,7 +40384,7 @@
         <v>1092</v>
       </c>
       <c r="L1282" s="57" t="str">
-        <f t="shared" si="140"/>
+        <f t="shared" si="141"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0420_Schu/0040_Sw_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -40313,7 +40399,7 @@
         <v>105</v>
       </c>
       <c r="L1283" s="57" t="str">
-        <f t="shared" si="139"/>
+        <f t="shared" si="140"/>
         <v/>
       </c>
     </row>
@@ -40387,7 +40473,7 @@
         <v>983</v>
       </c>
       <c r="L1290" s="57" t="str">
-        <f t="shared" ref="L1290:L1292" si="141">_xlfn.TEXTJOIN("", TRUE, D1290:J1290)</f>
+        <f t="shared" ref="L1290:L1292" si="142">_xlfn.TEXTJOIN("", TRUE, D1290:J1290)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0001_qbH-snw=f_01.png</v>
       </c>
     </row>
@@ -40408,7 +40494,7 @@
         <v>984</v>
       </c>
       <c r="L1291" s="57" t="str">
-        <f t="shared" si="141"/>
+        <f t="shared" si="142"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0010_qbH-snw=f_02.png</v>
       </c>
     </row>
@@ -40429,7 +40515,7 @@
         <v>985</v>
       </c>
       <c r="L1292" s="57" t="str">
-        <f t="shared" si="141"/>
+        <f t="shared" si="142"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0020_qbH-snw=f_03.png</v>
       </c>
     </row>
@@ -40459,7 +40545,7 @@
         <v>1092</v>
       </c>
       <c r="L1293" s="57" t="str">
-        <f t="shared" ref="L1293:L1300" si="142">_xlfn.TEXTJOIN("", TRUE, D1293:K1293)</f>
+        <f t="shared" ref="L1293:L1300" si="143">_xlfn.TEXTJOIN("", TRUE, D1293:K1293)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0030_qbH-snw=f_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -40489,7 +40575,7 @@
         <v>1092</v>
       </c>
       <c r="L1294" s="57" t="str">
-        <f t="shared" si="142"/>
+        <f t="shared" si="143"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0040_qbH-snw=f_MR_02.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -40519,7 +40605,7 @@
         <v>1092</v>
       </c>
       <c r="L1295" s="57" t="str">
-        <f t="shared" si="142"/>
+        <f t="shared" si="143"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0050_qbH-snw=f_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -40549,7 +40635,7 @@
         <v>1092</v>
       </c>
       <c r="L1296" s="57" t="str">
-        <f t="shared" si="142"/>
+        <f t="shared" si="143"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0060_qbH-snw=f_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -40579,7 +40665,7 @@
         <v>1092</v>
       </c>
       <c r="L1297" s="57" t="str">
-        <f t="shared" si="142"/>
+        <f t="shared" si="143"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0070_qbH-snw=f_GR_03.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -40609,7 +40695,7 @@
         <v>1092</v>
       </c>
       <c r="L1298" s="57" t="str">
-        <f t="shared" si="142"/>
+        <f t="shared" si="143"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0080_qbH-snw=f_GR_04.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -40642,7 +40728,7 @@
         <v>1092</v>
       </c>
       <c r="L1299" s="57" t="str">
-        <f t="shared" si="142"/>
+        <f t="shared" si="143"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/det/0001_qbH-snw=f_det_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -40675,7 +40761,7 @@
         <v>1092</v>
       </c>
       <c r="L1300" s="57" t="str">
-        <f t="shared" si="142"/>
+        <f t="shared" si="143"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/det/0010_qbH-snw=f_det_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -40758,7 +40844,7 @@
         <v>1092</v>
       </c>
       <c r="L1307" s="57" t="str">
-        <f t="shared" ref="L1307:L1311" si="143">_xlfn.TEXTJOIN("", TRUE, D1307:K1307)</f>
+        <f t="shared" ref="L1307:L1311" si="144">_xlfn.TEXTJOIN("", TRUE, D1307:K1307)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0440_Duamutef/0001_dwA-mw.t=f_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -40788,7 +40874,7 @@
         <v>1092</v>
       </c>
       <c r="L1308" s="57" t="str">
-        <f t="shared" si="143"/>
+        <f t="shared" si="144"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0440_Duamutef/0010_dwA-mw.t=f_AR_02.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -40818,7 +40904,7 @@
         <v>1092</v>
       </c>
       <c r="L1309" s="57" t="str">
-        <f t="shared" si="143"/>
+        <f t="shared" si="144"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0440_Duamutef/0020_dwA-mw.t=f_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -40848,7 +40934,7 @@
         <v>1092</v>
       </c>
       <c r="L1310" s="57" t="str">
-        <f t="shared" si="143"/>
+        <f t="shared" si="144"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0440_Duamutef/0030_dwA-mw.t=f_MR_02.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -40878,7 +40964,7 @@
         <v>1092</v>
       </c>
       <c r="L1311" s="57" t="str">
-        <f t="shared" si="143"/>
+        <f t="shared" si="144"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0440_Duamutef/0040_dwA-mw.t=f_MR_03.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -40893,7 +40979,7 @@
         <v>105</v>
       </c>
       <c r="L1312" s="57" t="str">
-        <f t="shared" ref="L1312" si="144">_xlfn.TEXTJOIN("", TRUE, D1312:J1312)</f>
+        <f t="shared" ref="L1312" si="145">_xlfn.TEXTJOIN("", TRUE, D1312:J1312)</f>
         <v/>
       </c>
     </row>
@@ -40976,7 +41062,7 @@
         <v>1092</v>
       </c>
       <c r="L1319" s="57" t="str">
-        <f t="shared" ref="L1319:L1329" si="145">_xlfn.TEXTJOIN("", TRUE, D1319:K1319)</f>
+        <f t="shared" ref="L1319:L1329" si="146">_xlfn.TEXTJOIN("", TRUE, D1319:K1319)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0001_DHwtj_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -41006,7 +41092,7 @@
         <v>1092</v>
       </c>
       <c r="L1320" s="57" t="str">
-        <f t="shared" si="145"/>
+        <f t="shared" si="146"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0010_DHwtj_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -41036,7 +41122,7 @@
         <v>1092</v>
       </c>
       <c r="L1321" s="57" t="str">
-        <f t="shared" si="145"/>
+        <f t="shared" si="146"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0020_DHwtj_MR_02.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -41066,7 +41152,7 @@
         <v>1092</v>
       </c>
       <c r="L1322" s="57" t="str">
-        <f t="shared" si="145"/>
+        <f t="shared" si="146"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0030_DHwtj_MR_03.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -41096,7 +41182,7 @@
         <v>1092</v>
       </c>
       <c r="L1323" s="57" t="str">
-        <f t="shared" si="145"/>
+        <f t="shared" si="146"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0040_DHwtj_MR_04.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -41126,7 +41212,7 @@
         <v>1092</v>
       </c>
       <c r="L1324" s="57" t="str">
-        <f t="shared" si="145"/>
+        <f t="shared" si="146"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0050_DHwtj_MR_05.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -41156,7 +41242,7 @@
         <v>1092</v>
       </c>
       <c r="L1325" s="57" t="str">
-        <f t="shared" si="145"/>
+        <f t="shared" si="146"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0060_DHwtj_SP_01.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -41186,7 +41272,7 @@
         <v>1092</v>
       </c>
       <c r="L1326" s="57" t="str">
-        <f t="shared" si="145"/>
+        <f t="shared" si="146"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0070_DHwtj_SP_02.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -41216,7 +41302,7 @@
         <v>1092</v>
       </c>
       <c r="L1327" s="57" t="str">
-        <f t="shared" si="145"/>
+        <f t="shared" si="146"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0080_DHwtj_SP-GR_01.png &lt;sup&gt;(Sp.; Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -41246,7 +41332,7 @@
         <v>1092</v>
       </c>
       <c r="L1328" s="57" t="str">
-        <f t="shared" si="145"/>
+        <f t="shared" si="146"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0090_DHwtj_SP-GR_02.png &lt;sup&gt;(Sp.; Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -41279,7 +41365,7 @@
         <v>1092</v>
       </c>
       <c r="L1329" s="57" t="str">
-        <f t="shared" si="145"/>
+        <f t="shared" si="146"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/det/0001_DHwtj_det_SP_01.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
       </c>
     </row>
@@ -41356,7 +41442,7 @@
         <v>111</v>
       </c>
       <c r="L1339" s="57" t="str">
-        <f t="shared" ref="L1339" si="146">_xlfn.TEXTJOIN("", TRUE, D1339:K1339)</f>
+        <f t="shared" ref="L1339" si="147">_xlfn.TEXTJOIN("", TRUE, D1339:K1339)</f>
         <v>03_Hieroglyphen-selten/F63_xnty_01.png</v>
       </c>
     </row>
@@ -41422,7 +41508,7 @@
         <v>111</v>
       </c>
       <c r="L1347" s="57" t="str">
-        <f t="shared" ref="L1347" si="147">_xlfn.TEXTJOIN("", TRUE, D1347:K1347)</f>
+        <f t="shared" ref="L1347" si="148">_xlfn.TEXTJOIN("", TRUE, D1347:K1347)</f>
         <v>03_Hieroglyphen-selten/N6B_nsw-bjt_01.png</v>
       </c>
     </row>
@@ -41488,7 +41574,7 @@
         <v>111</v>
       </c>
       <c r="L1351" s="57" t="str">
-        <f t="shared" ref="L1351" si="148">_xlfn.TEXTJOIN("", TRUE, D1351:K1351)</f>
+        <f t="shared" ref="L1351" si="149">_xlfn.TEXTJOIN("", TRUE, D1351:K1351)</f>
         <v>03_Hieroglyphen-selten/N102_jmn_01.png</v>
       </c>
     </row>
@@ -41526,4 +41612,145 @@
     <ignoredError sqref="L37 L1213 L1162" formula="1"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81889703-D8B6-7D4F-BE4B-112C79E1F253}">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="1" max="2" width="10.83203125" style="66"/>
+    <col min="3" max="3" width="25.6640625" style="66" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="10.83203125" style="66"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="67" customFormat="1">
+      <c r="A1" s="67" t="s">
+        <v>1645</v>
+      </c>
+      <c r="B1" s="67" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1" s="67" t="s">
+        <v>1646</v>
+      </c>
+      <c r="D1" s="67" t="s">
+        <v>1647</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="17">
+      <c r="A2" t="s">
+        <v>1648</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="68" t="s">
+        <v>1662</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1649</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="17">
+      <c r="A3" t="s">
+        <v>1648</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" s="68" t="s">
+        <v>1663</v>
+      </c>
+      <c r="D3" t="s">
+        <v>1650</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="17">
+      <c r="A4" t="s">
+        <v>1648</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" s="68" t="s">
+        <v>1664</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1651</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="17">
+      <c r="A5" t="s">
+        <v>1648</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5" s="68" t="s">
+        <v>1665</v>
+      </c>
+      <c r="D5" t="s">
+        <v>1652</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="17">
+      <c r="A6" t="s">
+        <v>1653</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" s="68" t="s">
+        <v>1654</v>
+      </c>
+      <c r="D6" t="s">
+        <v>1655</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="17">
+      <c r="A7" t="s">
+        <v>1653</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" s="68" t="s">
+        <v>1656</v>
+      </c>
+      <c r="D7" t="s">
+        <v>1657</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="17">
+      <c r="A8" t="s">
+        <v>1653</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" s="68" t="s">
+        <v>1658</v>
+      </c>
+      <c r="D8" t="s">
+        <v>1659</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="17">
+      <c r="A9" t="s">
+        <v>1653</v>
+      </c>
+      <c r="B9">
+        <v>4</v>
+      </c>
+      <c r="C9" s="68" t="s">
+        <v>1660</v>
+      </c>
+      <c r="D9" t="s">
+        <v>1661</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
changed order of formulas
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/MarkusKutschka/Documents/Arbeit/Inschriftenschluessel/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE2FD7E0-33E7-844E-9A73-1B47E614DF20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70C95CB1-89F1-4F4D-828E-C194544B0EB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="900" yWindow="660" windowWidth="22260" windowHeight="16200" activeTab="1" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
+    <workbookView xWindow="900" yWindow="660" windowWidth="18940" windowHeight="16200" activeTab="1" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
   </bookViews>
   <sheets>
     <sheet name="pages" sheetId="1" r:id="rId1"/>
@@ -6106,7 +6106,7 @@
         <v>61</v>
       </c>
       <c r="D3" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.2">
@@ -6120,7 +6120,7 @@
         <v>62</v>
       </c>
       <c r="D4" s="5">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.2">
@@ -6134,7 +6134,7 @@
         <v>63</v>
       </c>
       <c r="D5" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.2">
@@ -6162,7 +6162,7 @@
         <v>65</v>
       </c>
       <c r="D7" s="8">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
changed appearance of formula glyphlines
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/MarkusKutschka/Documents/Arbeit/Inschriftenschluessel/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7D1DCCD-60B5-504F-80E5-0DE429FB4C74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B554C84B-428E-5D43-A940-AEC4C0A362D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="900" yWindow="660" windowWidth="21260" windowHeight="16200" activeTab="4" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
+    <workbookView xWindow="-22120" yWindow="1540" windowWidth="21260" windowHeight="16200" activeTab="4" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
   </bookViews>
   <sheets>
     <sheet name="pages" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8040" uniqueCount="1685">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8026" uniqueCount="1685">
   <si>
     <t>page_id</t>
   </si>
@@ -5277,7 +5277,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -5410,7 +5410,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -9360,7 +9359,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="138" spans="1:11" ht="204" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:11" ht="221" x14ac:dyDescent="0.2">
       <c r="A138" s="13" t="s">
         <v>1257</v>
       </c>
@@ -9623,15 +9622,6 @@
       </c>
     </row>
     <row r="6" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B6" s="3">
-        <v>4</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>44</v>
-      </c>
       <c r="D6" s="3" t="s">
         <v>1545</v>
       </c>
@@ -9707,15 +9697,6 @@
       </c>
     </row>
     <row r="10" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" s="3">
-        <v>8</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>44</v>
-      </c>
       <c r="D10" s="3" t="s">
         <v>1545</v>
       </c>
@@ -10402,15 +10383,7 @@
       </c>
     </row>
     <row r="42" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="16" t="s">
-        <v>321</v>
-      </c>
-      <c r="B42" s="4">
-        <v>6</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="A42" s="16"/>
       <c r="D42" s="4" t="s">
         <v>1545</v>
       </c>
@@ -10483,15 +10456,7 @@
       </c>
     </row>
     <row r="46" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="16" t="s">
-        <v>321</v>
-      </c>
-      <c r="B46" s="4">
-        <v>10</v>
-      </c>
-      <c r="C46" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="A46" s="16"/>
       <c r="D46" s="4" t="s">
         <v>1545</v>
       </c>
@@ -11530,15 +11495,7 @@
       </c>
     </row>
     <row r="93" spans="1:14" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A93" s="18" t="s">
-        <v>356</v>
-      </c>
-      <c r="B93" s="5">
-        <v>8</v>
-      </c>
-      <c r="C93" s="5" t="s">
-        <v>44</v>
-      </c>
+      <c r="A93" s="18"/>
       <c r="D93" s="5" t="s">
         <v>1545</v>
       </c>
@@ -11661,15 +11618,7 @@
       </c>
     </row>
     <row r="99" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A99" s="18" t="s">
-        <v>356</v>
-      </c>
-      <c r="B99" s="5">
-        <v>14</v>
-      </c>
-      <c r="C99" s="5" t="s">
-        <v>44</v>
-      </c>
+      <c r="A99" s="18"/>
       <c r="D99" s="5" t="s">
         <v>1545</v>
       </c>
@@ -15504,20 +15453,11 @@
         <v>89</v>
       </c>
     </row>
-    <row r="288" spans="1:14" s="60" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A288" s="2" t="s">
-        <v>1037</v>
-      </c>
-      <c r="B288" s="60">
-        <v>10</v>
-      </c>
-      <c r="C288" s="60" t="s">
-        <v>44</v>
-      </c>
-      <c r="D288" s="60" t="s">
+    <row r="288" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="D288" s="2" t="s">
         <v>1545</v>
       </c>
-      <c r="N288" s="60" t="s">
+      <c r="N288" s="2" t="s">
         <v>89</v>
       </c>
     </row>

</xml_diff>